<commit_message>
ADAP 2023: Complete draft of budget and justification
</commit_message>
<xml_diff>
--- a/budget/BudgetDetails.xlsx
+++ b/budget/BudgetDetails.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kpenev/projects/git/proposals/TESS_EB_Bayesian_Proposal/budget/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD0DE066-2F13-A740-87FF-900045B32C9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C8E16A1-0861-394D-87AC-EF44119C9C37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="460" windowWidth="33600" windowHeight="20540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1594,33 +1594,53 @@
     <xf numFmtId="167" fontId="0" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="14" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="3" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1637,14 +1657,8 @@
     <xf numFmtId="49" fontId="4" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1656,31 +1670,29 @@
     <xf numFmtId="0" fontId="9" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="13" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="13" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1707,18 +1719,6 @@
     <xf numFmtId="0" fontId="11" fillId="12" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="12" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="12" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="15" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3035,15 +3035,15 @@
       <c r="D2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="199" t="s">
+      <c r="E2" s="235" t="s">
         <v>151</v>
       </c>
-      <c r="F2" s="199"/>
-      <c r="G2" s="199"/>
-      <c r="H2" s="199"/>
-      <c r="I2" s="199"/>
-      <c r="J2" s="199"/>
-      <c r="K2" s="199"/>
+      <c r="F2" s="235"/>
+      <c r="G2" s="235"/>
+      <c r="H2" s="235"/>
+      <c r="I2" s="235"/>
+      <c r="J2" s="235"/>
+      <c r="K2" s="235"/>
       <c r="L2" s="159"/>
       <c r="M2" s="159"/>
       <c r="N2" s="159"/>
@@ -3055,21 +3055,21 @@
       <c r="T2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="U2" s="200" t="s">
+      <c r="U2" s="236" t="s">
         <v>152</v>
       </c>
-      <c r="V2" s="201"/>
-      <c r="W2" s="201"/>
-      <c r="X2" s="201"/>
-      <c r="Y2" s="201"/>
-      <c r="Z2" s="201"/>
-      <c r="AA2" s="201"/>
-      <c r="AB2" s="201"/>
-      <c r="AC2" s="201"/>
-      <c r="AD2" s="201"/>
-      <c r="AE2" s="201"/>
-      <c r="AF2" s="201"/>
-      <c r="AG2" s="201"/>
+      <c r="V2" s="237"/>
+      <c r="W2" s="237"/>
+      <c r="X2" s="237"/>
+      <c r="Y2" s="237"/>
+      <c r="Z2" s="237"/>
+      <c r="AA2" s="237"/>
+      <c r="AB2" s="237"/>
+      <c r="AC2" s="237"/>
+      <c r="AD2" s="237"/>
+      <c r="AE2" s="237"/>
+      <c r="AF2" s="237"/>
+      <c r="AG2" s="237"/>
       <c r="AH2" s="159"/>
       <c r="AJ2" s="159"/>
       <c r="AK2" s="159"/>
@@ -3164,15 +3164,15 @@
       <c r="D4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="199" t="s">
+      <c r="E4" s="235" t="s">
         <v>154</v>
       </c>
-      <c r="F4" s="199"/>
-      <c r="G4" s="199"/>
-      <c r="H4" s="199"/>
-      <c r="I4" s="199"/>
-      <c r="J4" s="199"/>
-      <c r="K4" s="199"/>
+      <c r="F4" s="235"/>
+      <c r="G4" s="235"/>
+      <c r="H4" s="235"/>
+      <c r="I4" s="235"/>
+      <c r="J4" s="235"/>
+      <c r="K4" s="235"/>
       <c r="L4" s="3"/>
       <c r="M4" s="3"/>
       <c r="N4" s="3"/>
@@ -3185,24 +3185,24 @@
         <v>3</v>
       </c>
       <c r="U4" s="3"/>
-      <c r="V4" s="206">
+      <c r="V4" s="202">
         <v>43965</v>
       </c>
-      <c r="W4" s="206"/>
-      <c r="X4" s="206"/>
+      <c r="W4" s="202"/>
+      <c r="X4" s="202"/>
       <c r="Y4" s="3"/>
       <c r="Z4" s="3"/>
-      <c r="AA4" s="256" t="s">
+      <c r="AA4" s="201" t="s">
         <v>155</v>
       </c>
-      <c r="AB4" s="256"/>
-      <c r="AC4" s="256"/>
+      <c r="AB4" s="201"/>
+      <c r="AC4" s="201"/>
       <c r="AD4" s="159"/>
-      <c r="AE4" s="206">
+      <c r="AE4" s="202">
         <v>44694</v>
       </c>
-      <c r="AF4" s="206"/>
-      <c r="AG4" s="206"/>
+      <c r="AF4" s="202"/>
+      <c r="AG4" s="202"/>
       <c r="AH4" s="159"/>
       <c r="AJ4" s="7"/>
       <c r="AK4" s="7"/>
@@ -3212,11 +3212,11 @@
       <c r="AR4" s="159"/>
       <c r="AS4" s="159"/>
       <c r="AT4" s="159"/>
-      <c r="AU4" s="255" t="s">
+      <c r="AU4" s="233" t="s">
         <v>4</v>
       </c>
-      <c r="AV4" s="207"/>
-      <c r="AW4" s="207"/>
+      <c r="AV4" s="234"/>
+      <c r="AW4" s="234"/>
       <c r="AX4" s="159"/>
       <c r="AY4" s="159"/>
       <c r="AZ4" s="159"/>
@@ -3278,10 +3278,10 @@
       <c r="AU5" s="159"/>
       <c r="AV5" s="159"/>
       <c r="AW5" s="159"/>
-      <c r="AX5" s="257"/>
-      <c r="AY5" s="257"/>
-      <c r="AZ5" s="257"/>
-      <c r="BA5" s="258"/>
+      <c r="AX5" s="199"/>
+      <c r="AY5" s="199"/>
+      <c r="AZ5" s="199"/>
+      <c r="BA5" s="200"/>
       <c r="BB5" s="3"/>
       <c r="BC5" s="5"/>
       <c r="BD5" s="5"/>
@@ -3371,49 +3371,49 @@
       <c r="N7" s="14"/>
       <c r="O7" s="14"/>
       <c r="P7" s="14"/>
-      <c r="Q7" s="202" t="s">
+      <c r="Q7" s="226" t="s">
         <v>97</v>
       </c>
-      <c r="R7" s="219"/>
-      <c r="S7" s="219"/>
+      <c r="R7" s="227"/>
+      <c r="S7" s="227"/>
       <c r="T7" s="14"/>
       <c r="U7" s="14"/>
-      <c r="V7" s="202" t="s">
+      <c r="V7" s="226" t="s">
         <v>98</v>
       </c>
-      <c r="W7" s="203"/>
-      <c r="X7" s="203"/>
-      <c r="Y7" s="204"/>
-      <c r="Z7" s="205"/>
+      <c r="W7" s="230"/>
+      <c r="X7" s="230"/>
+      <c r="Y7" s="231"/>
+      <c r="Z7" s="232"/>
       <c r="AA7" s="14"/>
       <c r="AB7" s="14"/>
-      <c r="AC7" s="202" t="s">
+      <c r="AC7" s="226" t="s">
         <v>99</v>
       </c>
-      <c r="AD7" s="203"/>
-      <c r="AE7" s="203"/>
-      <c r="AF7" s="204"/>
-      <c r="AG7" s="205"/>
+      <c r="AD7" s="230"/>
+      <c r="AE7" s="230"/>
+      <c r="AF7" s="231"/>
+      <c r="AG7" s="232"/>
       <c r="AH7" s="14"/>
       <c r="AI7" s="14"/>
       <c r="AJ7" s="14"/>
       <c r="AK7" s="14"/>
       <c r="AL7" s="14"/>
-      <c r="AM7" s="202" t="s">
+      <c r="AM7" s="226" t="s">
         <v>6</v>
       </c>
-      <c r="AN7" s="204"/>
-      <c r="AO7" s="205"/>
+      <c r="AN7" s="231"/>
+      <c r="AO7" s="232"/>
       <c r="AP7" s="14"/>
       <c r="AQ7" s="14"/>
       <c r="AR7" s="14"/>
       <c r="AS7" s="14"/>
       <c r="AT7" s="14"/>
-      <c r="AU7" s="202" t="s">
+      <c r="AU7" s="226" t="s">
         <v>7</v>
       </c>
-      <c r="AV7" s="204"/>
-      <c r="AW7" s="205"/>
+      <c r="AV7" s="231"/>
+      <c r="AW7" s="232"/>
       <c r="AX7" s="14"/>
       <c r="AY7" s="14"/>
       <c r="AZ7" s="15"/>
@@ -3491,12 +3491,12 @@
         <v>8</v>
       </c>
       <c r="B9" s="3"/>
-      <c r="C9" s="222" t="s">
+      <c r="C9" s="205" t="s">
         <v>9</v>
       </c>
-      <c r="D9" s="216"/>
-      <c r="E9" s="217"/>
-      <c r="F9" s="218"/>
+      <c r="D9" s="206"/>
+      <c r="E9" s="207"/>
+      <c r="F9" s="208"/>
       <c r="G9" s="23"/>
       <c r="H9" s="23"/>
       <c r="I9" s="23"/>
@@ -3505,7 +3505,7 @@
       <c r="L9" s="24"/>
       <c r="M9" s="25"/>
       <c r="N9" s="26"/>
-      <c r="O9" s="223" t="s">
+      <c r="O9" s="213" t="s">
         <v>10</v>
       </c>
       <c r="P9" s="3"/>
@@ -3514,7 +3514,7 @@
       <c r="S9" s="3"/>
       <c r="T9" s="27"/>
       <c r="U9" s="28"/>
-      <c r="V9" s="223" t="s">
+      <c r="V9" s="213" t="s">
         <v>10</v>
       </c>
       <c r="W9" s="3"/>
@@ -3523,7 +3523,7 @@
       <c r="Z9" s="3"/>
       <c r="AA9" s="27"/>
       <c r="AB9" s="28"/>
-      <c r="AC9" s="223" t="s">
+      <c r="AC9" s="213" t="s">
         <v>10</v>
       </c>
       <c r="AD9" s="3"/>
@@ -3533,7 +3533,7 @@
       <c r="AH9" s="27"/>
       <c r="AI9" s="28"/>
       <c r="AJ9" s="3"/>
-      <c r="AK9" s="223" t="s">
+      <c r="AK9" s="213" t="s">
         <v>10</v>
       </c>
       <c r="AL9" s="3"/>
@@ -3543,7 +3543,7 @@
       <c r="AP9" s="27"/>
       <c r="AQ9" s="28"/>
       <c r="AR9" s="3"/>
-      <c r="AS9" s="223" t="s">
+      <c r="AS9" s="213" t="s">
         <v>10</v>
       </c>
       <c r="AT9" s="3"/>
@@ -3552,7 +3552,7 @@
       <c r="AW9" s="3"/>
       <c r="AX9" s="27"/>
       <c r="AY9" s="29"/>
-      <c r="AZ9" s="223" t="s">
+      <c r="AZ9" s="213" t="s">
         <v>11</v>
       </c>
       <c r="BA9" s="17"/>
@@ -3588,7 +3588,7 @@
       </c>
       <c r="M10" s="25"/>
       <c r="N10" s="26"/>
-      <c r="O10" s="224"/>
+      <c r="O10" s="214"/>
       <c r="P10" s="33"/>
       <c r="Q10" s="32" t="s">
         <v>17</v>
@@ -3599,7 +3599,7 @@
       </c>
       <c r="T10" s="35"/>
       <c r="U10" s="36"/>
-      <c r="V10" s="224"/>
+      <c r="V10" s="214"/>
       <c r="W10" s="33"/>
       <c r="X10" s="32" t="s">
         <v>17</v>
@@ -3610,7 +3610,7 @@
       </c>
       <c r="AA10" s="35"/>
       <c r="AB10" s="36"/>
-      <c r="AC10" s="224"/>
+      <c r="AC10" s="214"/>
       <c r="AD10" s="33"/>
       <c r="AE10" s="32" t="s">
         <v>17</v>
@@ -3622,7 +3622,7 @@
       <c r="AH10" s="35"/>
       <c r="AI10" s="36"/>
       <c r="AJ10" s="33"/>
-      <c r="AK10" s="224"/>
+      <c r="AK10" s="214"/>
       <c r="AL10" s="33"/>
       <c r="AM10" s="32" t="s">
         <v>17</v>
@@ -3634,7 +3634,7 @@
       <c r="AP10" s="35"/>
       <c r="AQ10" s="36"/>
       <c r="AR10" s="33"/>
-      <c r="AS10" s="224"/>
+      <c r="AS10" s="214"/>
       <c r="AT10" s="33"/>
       <c r="AU10" s="32" t="s">
         <v>17</v>
@@ -3645,7 +3645,7 @@
       </c>
       <c r="AX10" s="35"/>
       <c r="AY10" s="38"/>
-      <c r="AZ10" s="225"/>
+      <c r="AZ10" s="215"/>
       <c r="BA10" s="17"/>
       <c r="BB10" s="21"/>
       <c r="BC10" s="3"/>
@@ -3659,10 +3659,10 @@
       <c r="B11" s="39" t="s">
         <v>19</v>
       </c>
-      <c r="C11" s="226" t="s">
+      <c r="C11" s="216" t="s">
         <v>153</v>
       </c>
-      <c r="D11" s="227"/>
+      <c r="D11" s="217"/>
       <c r="E11" s="40"/>
       <c r="F11" s="41">
         <v>11712.89</v>
@@ -3754,7 +3754,7 @@
       <c r="AX11" s="50"/>
       <c r="AY11" s="53"/>
       <c r="AZ11" s="168">
-        <f>SUM(S11+Z11+AG11+AO11+AW11)</f>
+        <f t="shared" ref="AZ11:AZ16" si="5">SUM(S11+Z11+AG11+AO11+AW11)</f>
         <v>23777.166700000002</v>
       </c>
       <c r="BA11" s="17"/>
@@ -3770,10 +3770,10 @@
       <c r="B12" s="39" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="220" t="s">
+      <c r="C12" s="228" t="s">
         <v>156</v>
       </c>
-      <c r="D12" s="221"/>
+      <c r="D12" s="229"/>
       <c r="E12" s="40"/>
       <c r="F12" s="54">
         <v>0</v>
@@ -3865,7 +3865,7 @@
       <c r="AX12" s="50"/>
       <c r="AY12" s="53"/>
       <c r="AZ12" s="168">
-        <f>SUM(S12+Z12+AG12+AO12+AW12)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="BA12" s="17"/>
@@ -3881,10 +3881,10 @@
       <c r="B13" s="39" t="s">
         <v>21</v>
       </c>
-      <c r="C13" s="220" t="s">
+      <c r="C13" s="228" t="s">
         <v>107</v>
       </c>
-      <c r="D13" s="221"/>
+      <c r="D13" s="229"/>
       <c r="E13" s="40"/>
       <c r="F13" s="54">
         <v>0</v>
@@ -3976,7 +3976,7 @@
       <c r="AX13" s="50"/>
       <c r="AY13" s="53"/>
       <c r="AZ13" s="168">
-        <f>SUM(S13+Z13+AG13+AO13+AW13)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="BA13" s="17"/>
@@ -3992,10 +3992,10 @@
       <c r="B14" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="C14" s="220" t="s">
+      <c r="C14" s="228" t="s">
         <v>108</v>
       </c>
-      <c r="D14" s="221"/>
+      <c r="D14" s="229"/>
       <c r="E14" s="40"/>
       <c r="F14" s="54">
         <v>0</v>
@@ -4087,7 +4087,7 @@
       <c r="AX14" s="50"/>
       <c r="AY14" s="53"/>
       <c r="AZ14" s="168">
-        <f>SUM(S14+Z14+AG14+AO14+AW14)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="BA14" s="17"/>
@@ -4103,10 +4103,10 @@
       <c r="B15" s="39" t="s">
         <v>23</v>
       </c>
-      <c r="C15" s="208" t="s">
+      <c r="C15" s="218" t="s">
         <v>109</v>
       </c>
-      <c r="D15" s="209"/>
+      <c r="D15" s="219"/>
       <c r="E15" s="40"/>
       <c r="F15" s="54">
         <v>0</v>
@@ -4198,7 +4198,7 @@
       <c r="AX15" s="50"/>
       <c r="AY15" s="53"/>
       <c r="AZ15" s="168">
-        <f>SUM(S15+Z15+AG15+AO15+AW15)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="BA15" s="17"/>
@@ -4214,10 +4214,10 @@
       <c r="B16" s="39" t="s">
         <v>24</v>
       </c>
-      <c r="C16" s="210" t="s">
+      <c r="C16" s="220" t="s">
         <v>36</v>
       </c>
-      <c r="D16" s="211"/>
+      <c r="D16" s="221"/>
       <c r="E16" s="40"/>
       <c r="F16" s="59">
         <v>0</v>
@@ -4309,7 +4309,7 @@
       <c r="AX16" s="50"/>
       <c r="AY16" s="53"/>
       <c r="AZ16" s="169">
-        <f>SUM(S16+Z16+AG16+AO16+AW16)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="BA16" s="17"/>
@@ -4466,11 +4466,11 @@
       <c r="A19" s="81" t="s">
         <v>26</v>
       </c>
-      <c r="B19" s="212" t="s">
+      <c r="B19" s="222" t="s">
         <v>27</v>
       </c>
-      <c r="C19" s="213"/>
-      <c r="D19" s="214"/>
+      <c r="C19" s="223"/>
+      <c r="D19" s="224"/>
       <c r="E19" s="3"/>
       <c r="F19" s="32" t="s">
         <v>13</v>
@@ -4633,7 +4633,7 @@
       <c r="AX20" s="87"/>
       <c r="AY20" s="88"/>
       <c r="AZ20" s="168">
-        <f>SUM(S20+Z20+AG20+AO20+AW20)</f>
+        <f t="shared" ref="AZ20:AZ25" si="6">SUM(S20+Z20+AG20+AO20+AW20)</f>
         <v>0</v>
       </c>
       <c r="BA20" s="17"/>
@@ -4678,7 +4678,7 @@
       </c>
       <c r="R21" s="86"/>
       <c r="S21" s="165">
-        <f t="shared" ref="S21:S25" si="5">(IF(Q21&gt;0,Q21*$F21*$J21*(1+$H$6)^0,0))</f>
+        <f t="shared" ref="S21:S25" si="7">(IF(Q21&gt;0,Q21*$F21*$J21*(1+$H$6)^0,0))</f>
         <v>0</v>
       </c>
       <c r="T21" s="87"/>
@@ -4690,7 +4690,7 @@
       </c>
       <c r="Y21" s="88"/>
       <c r="Z21" s="165">
-        <f t="shared" ref="Z21:Z25" si="6">(IF(X21&gt;0,X21*$F21*$J21*(1+$H$6)^1,0))</f>
+        <f t="shared" ref="Z21:Z25" si="8">(IF(X21&gt;0,X21*$F21*$J21*(1+$H$6)^1,0))</f>
         <v>0</v>
       </c>
       <c r="AA21" s="87"/>
@@ -4702,7 +4702,7 @@
       </c>
       <c r="AF21" s="88"/>
       <c r="AG21" s="165">
-        <f t="shared" ref="AG21:AG25" si="7">(IF(AE21&gt;0,AE21*$F21*$J21*(1+$H$6)^2,0))</f>
+        <f t="shared" ref="AG21:AG25" si="9">(IF(AE21&gt;0,AE21*$F21*$J21*(1+$H$6)^2,0))</f>
         <v>0</v>
       </c>
       <c r="AH21" s="87"/>
@@ -4715,7 +4715,7 @@
       </c>
       <c r="AN21" s="88"/>
       <c r="AO21" s="165">
-        <f t="shared" ref="AO21:AO25" si="8">(IF(AM21&gt;0,AM21*$F21*$J21*(1+$H$6)^3,0))</f>
+        <f t="shared" ref="AO21:AO25" si="10">(IF(AM21&gt;0,AM21*$F21*$J21*(1+$H$6)^3,0))</f>
         <v>0</v>
       </c>
       <c r="AP21" s="87"/>
@@ -4728,13 +4728,13 @@
       </c>
       <c r="AV21" s="88"/>
       <c r="AW21" s="165">
-        <f t="shared" ref="AW21:AW25" si="9">(IF(AU21&gt;0,AU21*$F21*$J21*(1+$H$6)^4,0))</f>
+        <f t="shared" ref="AW21:AW25" si="11">(IF(AU21&gt;0,AU21*$F21*$J21*(1+$H$6)^4,0))</f>
         <v>0</v>
       </c>
       <c r="AX21" s="87"/>
       <c r="AY21" s="88"/>
       <c r="AZ21" s="168">
-        <f>SUM(S21+Z21+AG21+AO21+AW21)</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="BA21" s="17"/>
@@ -4758,7 +4758,7 @@
       </c>
       <c r="E22" s="66"/>
       <c r="F22" s="54">
-        <v>2200</v>
+        <v>2400</v>
       </c>
       <c r="G22" s="53"/>
       <c r="H22" s="178"/>
@@ -4779,8 +4779,8 @@
       </c>
       <c r="R22" s="86"/>
       <c r="S22" s="165">
-        <f t="shared" si="5"/>
-        <v>26400</v>
+        <f t="shared" si="7"/>
+        <v>28800</v>
       </c>
       <c r="T22" s="87"/>
       <c r="U22" s="88"/>
@@ -4791,8 +4791,8 @@
       </c>
       <c r="Y22" s="88"/>
       <c r="Z22" s="165">
-        <f t="shared" si="6"/>
-        <v>27192</v>
+        <f t="shared" si="8"/>
+        <v>29664</v>
       </c>
       <c r="AA22" s="87"/>
       <c r="AB22" s="88"/>
@@ -4803,7 +4803,7 @@
       </c>
       <c r="AF22" s="88"/>
       <c r="AG22" s="165">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="AH22" s="87"/>
@@ -4816,7 +4816,7 @@
       </c>
       <c r="AN22" s="88"/>
       <c r="AO22" s="165">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="AP22" s="87"/>
@@ -4829,14 +4829,14 @@
       </c>
       <c r="AV22" s="88"/>
       <c r="AW22" s="165">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="AX22" s="87"/>
       <c r="AY22" s="88"/>
       <c r="AZ22" s="168">
-        <f>SUM(S22+Z22+AG22+AO22+AW22)</f>
-        <v>53592</v>
+        <f t="shared" si="6"/>
+        <v>58464</v>
       </c>
       <c r="BA22" s="17"/>
       <c r="BB22" s="36"/>
@@ -4880,7 +4880,7 @@
       </c>
       <c r="R23" s="86"/>
       <c r="S23" s="165">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="T23" s="87"/>
@@ -4892,7 +4892,7 @@
       </c>
       <c r="Y23" s="88"/>
       <c r="Z23" s="165">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="AA23" s="87"/>
@@ -4904,7 +4904,7 @@
       </c>
       <c r="AF23" s="88"/>
       <c r="AG23" s="165">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="AH23" s="87"/>
@@ -4917,7 +4917,7 @@
       </c>
       <c r="AN23" s="88"/>
       <c r="AO23" s="165">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="AP23" s="87"/>
@@ -4930,13 +4930,13 @@
       </c>
       <c r="AV23" s="88"/>
       <c r="AW23" s="165">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="AX23" s="87"/>
       <c r="AY23" s="88"/>
       <c r="AZ23" s="168">
-        <f>SUM(S23+Z23+AG23+AO23+AW23)</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="BA23" s="17"/>
@@ -4981,7 +4981,7 @@
       </c>
       <c r="R24" s="86"/>
       <c r="S24" s="165">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="T24" s="87"/>
@@ -4993,7 +4993,7 @@
       </c>
       <c r="Y24" s="88"/>
       <c r="Z24" s="165">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="AA24" s="87"/>
@@ -5005,7 +5005,7 @@
       </c>
       <c r="AF24" s="88"/>
       <c r="AG24" s="165">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="AH24" s="87"/>
@@ -5018,7 +5018,7 @@
       </c>
       <c r="AN24" s="88"/>
       <c r="AO24" s="165">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="AP24" s="87"/>
@@ -5031,13 +5031,13 @@
       </c>
       <c r="AV24" s="88"/>
       <c r="AW24" s="165">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="AX24" s="87"/>
       <c r="AY24" s="88"/>
       <c r="AZ24" s="168">
-        <f>SUM(S24+Z24+AG24+AO24+AW24)</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="BA24" s="17"/>
@@ -5082,7 +5082,7 @@
       </c>
       <c r="R25" s="86"/>
       <c r="S25" s="165">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="T25" s="87"/>
@@ -5094,7 +5094,7 @@
       </c>
       <c r="Y25" s="88"/>
       <c r="Z25" s="165">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="AA25" s="87"/>
@@ -5106,7 +5106,7 @@
       </c>
       <c r="AF25" s="88"/>
       <c r="AG25" s="165">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="AH25" s="87"/>
@@ -5119,7 +5119,7 @@
       </c>
       <c r="AN25" s="88"/>
       <c r="AO25" s="165">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="AP25" s="87"/>
@@ -5132,13 +5132,13 @@
       </c>
       <c r="AV25" s="88"/>
       <c r="AW25" s="165">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="AX25" s="87"/>
       <c r="AY25" s="88"/>
       <c r="AZ25" s="169">
-        <f>SUM(S25+Z25+AG25+AO25+AW25)</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="BA25" s="17"/>
@@ -5172,7 +5172,7 @@
       <c r="R26" s="69"/>
       <c r="S26" s="170">
         <f>SUM(S20:S25)</f>
-        <v>26400</v>
+        <v>28800</v>
       </c>
       <c r="T26" s="89"/>
       <c r="U26" s="90"/>
@@ -5182,7 +5182,7 @@
       <c r="Y26" s="92"/>
       <c r="Z26" s="170">
         <f>SUM(Z20:Z25)</f>
-        <v>27192</v>
+        <v>29664</v>
       </c>
       <c r="AA26" s="89"/>
       <c r="AB26" s="90"/>
@@ -5220,7 +5220,7 @@
       <c r="AY26" s="90"/>
       <c r="AZ26" s="167">
         <f>SUM(AZ20:AZ25)</f>
-        <v>53592</v>
+        <v>58464</v>
       </c>
       <c r="BA26" s="17"/>
       <c r="BB26" s="21"/>
@@ -5314,7 +5314,7 @@
       <c r="R28" s="69"/>
       <c r="S28" s="171">
         <f>S17+S26</f>
-        <v>38112.89</v>
+        <v>40512.89</v>
       </c>
       <c r="T28" s="89"/>
       <c r="U28" s="90"/>
@@ -5324,7 +5324,7 @@
       <c r="Y28" s="92"/>
       <c r="Z28" s="171">
         <f>Z17+Z26</f>
-        <v>39256.276700000002</v>
+        <v>41728.276700000002</v>
       </c>
       <c r="AA28" s="89"/>
       <c r="AB28" s="90"/>
@@ -5362,7 +5362,7 @@
       <c r="AY28" s="90"/>
       <c r="AZ28" s="168">
         <f>AZ17+AZ26</f>
-        <v>77369.166700000002</v>
+        <v>82241.166700000002</v>
       </c>
       <c r="BA28" s="17"/>
       <c r="BB28" s="21"/>
@@ -5437,13 +5437,13 @@
       <c r="A30" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="B30" s="215" t="s">
+      <c r="B30" s="225" t="s">
         <v>35</v>
       </c>
-      <c r="C30" s="216"/>
-      <c r="D30" s="217"/>
-      <c r="E30" s="217"/>
-      <c r="F30" s="218"/>
+      <c r="C30" s="206"/>
+      <c r="D30" s="207"/>
+      <c r="E30" s="207"/>
+      <c r="F30" s="208"/>
       <c r="G30" s="23"/>
       <c r="H30" s="23"/>
       <c r="I30" s="23"/>
@@ -5509,7 +5509,7 @@
       <c r="D31" s="3"/>
       <c r="E31" s="3"/>
       <c r="F31" s="30" t="str">
-        <f t="shared" ref="F31:F36" si="10">C11</f>
+        <f t="shared" ref="F31:F36" si="12">C11</f>
         <v>PI Kaloyan Penev</v>
       </c>
       <c r="G31" s="30"/>
@@ -5525,7 +5525,7 @@
       <c r="Q31" s="3"/>
       <c r="R31" s="3"/>
       <c r="S31" s="168">
-        <f t="shared" ref="S31:S36" si="11">S11*L11</f>
+        <f t="shared" ref="S31:S36" si="13">S11*L11</f>
         <v>3748.1248000000001</v>
       </c>
       <c r="T31" s="50"/>
@@ -5535,7 +5535,7 @@
       <c r="X31" s="3"/>
       <c r="Y31" s="102"/>
       <c r="Z31" s="168">
-        <f t="shared" ref="Z31:Z36" si="12">Z11*L11</f>
+        <f t="shared" ref="Z31:Z36" si="14">Z11*L11</f>
         <v>3860.5685440000002</v>
       </c>
       <c r="AA31" s="50"/>
@@ -5545,7 +5545,7 @@
       <c r="AE31" s="3"/>
       <c r="AF31" s="102"/>
       <c r="AG31" s="168">
-        <f t="shared" ref="AG31:AG36" si="13">AG11*L11</f>
+        <f t="shared" ref="AG31:AG36" si="15">AG11*L11</f>
         <v>0</v>
       </c>
       <c r="AH31" s="50"/>
@@ -5556,7 +5556,7 @@
       <c r="AM31" s="102"/>
       <c r="AN31" s="102"/>
       <c r="AO31" s="168">
-        <f t="shared" ref="AO31:AO36" si="14">AO11*L11</f>
+        <f t="shared" ref="AO31:AO36" si="16">AO11*L11</f>
         <v>0</v>
       </c>
       <c r="AP31" s="50"/>
@@ -5567,13 +5567,13 @@
       <c r="AU31" s="102"/>
       <c r="AV31" s="102"/>
       <c r="AW31" s="168">
-        <f t="shared" ref="AW31:AW36" si="15">AW11*L11</f>
+        <f t="shared" ref="AW31:AW36" si="17">AW11*L11</f>
         <v>0</v>
       </c>
       <c r="AX31" s="50"/>
       <c r="AY31" s="53"/>
       <c r="AZ31" s="168">
-        <f>SUM(S31+Z31+AG31+AO31+AW31)</f>
+        <f t="shared" ref="AZ31:AZ42" si="18">SUM(S31+Z31+AG31+AO31+AW31)</f>
         <v>7608.6933440000003</v>
       </c>
       <c r="BA31" s="17"/>
@@ -5595,7 +5595,7 @@
       <c r="D32" s="3"/>
       <c r="E32" s="3"/>
       <c r="F32" s="30" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>Co1</v>
       </c>
       <c r="G32" s="30"/>
@@ -5611,7 +5611,7 @@
       <c r="Q32" s="3"/>
       <c r="R32" s="3"/>
       <c r="S32" s="168">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="T32" s="50"/>
@@ -5621,7 +5621,7 @@
       <c r="X32" s="3"/>
       <c r="Y32" s="102"/>
       <c r="Z32" s="168">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="AA32" s="50"/>
@@ -5631,7 +5631,7 @@
       <c r="AE32" s="3"/>
       <c r="AF32" s="102"/>
       <c r="AG32" s="168">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="AH32" s="50"/>
@@ -5642,7 +5642,7 @@
       <c r="AM32" s="102"/>
       <c r="AN32" s="102"/>
       <c r="AO32" s="168">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="AP32" s="50"/>
@@ -5653,13 +5653,13 @@
       <c r="AU32" s="102"/>
       <c r="AV32" s="102"/>
       <c r="AW32" s="168">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="AX32" s="50"/>
       <c r="AY32" s="53"/>
       <c r="AZ32" s="168">
-        <f>SUM(S32+Z32+AG32+AO32+AW32)</f>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="BA32" s="17"/>
@@ -5681,7 +5681,7 @@
       <c r="D33" s="3"/>
       <c r="E33" s="3"/>
       <c r="F33" s="30" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>Co2</v>
       </c>
       <c r="G33" s="30"/>
@@ -5697,7 +5697,7 @@
       <c r="Q33" s="3"/>
       <c r="R33" s="3"/>
       <c r="S33" s="168">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="T33" s="50"/>
@@ -5707,7 +5707,7 @@
       <c r="X33" s="3"/>
       <c r="Y33" s="102"/>
       <c r="Z33" s="168">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="AA33" s="50"/>
@@ -5717,7 +5717,7 @@
       <c r="AE33" s="3"/>
       <c r="AF33" s="102"/>
       <c r="AG33" s="168">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="AH33" s="50"/>
@@ -5728,7 +5728,7 @@
       <c r="AM33" s="102"/>
       <c r="AN33" s="102"/>
       <c r="AO33" s="168">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="AP33" s="50"/>
@@ -5739,13 +5739,13 @@
       <c r="AU33" s="102"/>
       <c r="AV33" s="102"/>
       <c r="AW33" s="168">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="AX33" s="50"/>
       <c r="AY33" s="53"/>
       <c r="AZ33" s="168">
-        <f>SUM(S33+Z33+AG33+AO33+AW33)</f>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="BA33" s="17"/>
@@ -5767,7 +5767,7 @@
       <c r="D34" s="3"/>
       <c r="E34" s="3"/>
       <c r="F34" s="30" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>Co3</v>
       </c>
       <c r="G34" s="30"/>
@@ -5783,7 +5783,7 @@
       <c r="Q34" s="3"/>
       <c r="R34" s="3"/>
       <c r="S34" s="168">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="T34" s="50"/>
@@ -5793,7 +5793,7 @@
       <c r="X34" s="3"/>
       <c r="Y34" s="102"/>
       <c r="Z34" s="168">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="AA34" s="50"/>
@@ -5803,7 +5803,7 @@
       <c r="AE34" s="3"/>
       <c r="AF34" s="102"/>
       <c r="AG34" s="168">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="AH34" s="50"/>
@@ -5814,7 +5814,7 @@
       <c r="AM34" s="102"/>
       <c r="AN34" s="102"/>
       <c r="AO34" s="168">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="AP34" s="50"/>
@@ -5825,13 +5825,13 @@
       <c r="AU34" s="102"/>
       <c r="AV34" s="102"/>
       <c r="AW34" s="168">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="AX34" s="50"/>
       <c r="AY34" s="53"/>
       <c r="AZ34" s="168">
-        <f>SUM(S34+Z34+AG34+AO34+AW34)</f>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="BA34" s="17"/>
@@ -5853,7 +5853,7 @@
       <c r="D35" s="3"/>
       <c r="E35" s="3"/>
       <c r="F35" s="30" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>Co4</v>
       </c>
       <c r="G35" s="30"/>
@@ -5869,7 +5869,7 @@
       <c r="Q35" s="3"/>
       <c r="R35" s="3"/>
       <c r="S35" s="168">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="T35" s="50"/>
@@ -5879,7 +5879,7 @@
       <c r="X35" s="3"/>
       <c r="Y35" s="102"/>
       <c r="Z35" s="168">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="AA35" s="50"/>
@@ -5889,7 +5889,7 @@
       <c r="AE35" s="3"/>
       <c r="AF35" s="102"/>
       <c r="AG35" s="168">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="AH35" s="50"/>
@@ -5900,7 +5900,7 @@
       <c r="AM35" s="102"/>
       <c r="AN35" s="102"/>
       <c r="AO35" s="168">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="AP35" s="50"/>
@@ -5911,13 +5911,13 @@
       <c r="AU35" s="102"/>
       <c r="AV35" s="102"/>
       <c r="AW35" s="168">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="AX35" s="50"/>
       <c r="AY35" s="53"/>
       <c r="AZ35" s="168">
-        <f>SUM(S35+Z35+AG35+AO35+AW35)</f>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="BA35" s="17"/>
@@ -5939,7 +5939,7 @@
       <c r="D36" s="3"/>
       <c r="E36" s="3"/>
       <c r="F36" s="30" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>Senior Personnel</v>
       </c>
       <c r="G36" s="30"/>
@@ -5955,7 +5955,7 @@
       <c r="Q36" s="3"/>
       <c r="R36" s="3"/>
       <c r="S36" s="168">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="T36" s="50"/>
@@ -5965,7 +5965,7 @@
       <c r="X36" s="3"/>
       <c r="Y36" s="102"/>
       <c r="Z36" s="168">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="AA36" s="50"/>
@@ -5975,7 +5975,7 @@
       <c r="AE36" s="3"/>
       <c r="AF36" s="102"/>
       <c r="AG36" s="168">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="AH36" s="50"/>
@@ -5986,7 +5986,7 @@
       <c r="AM36" s="102"/>
       <c r="AN36" s="102"/>
       <c r="AO36" s="168">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="AP36" s="50"/>
@@ -5997,13 +5997,13 @@
       <c r="AU36" s="102"/>
       <c r="AV36" s="102"/>
       <c r="AW36" s="168">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="AX36" s="50"/>
       <c r="AY36" s="53"/>
       <c r="AZ36" s="168">
-        <f>SUM(S36+Z36+AG36+AO36+AW36)</f>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="BA36" s="17"/>
@@ -6038,7 +6038,7 @@
       <c r="Q37" s="3"/>
       <c r="R37" s="3"/>
       <c r="S37" s="168">
-        <f t="shared" ref="S37:S42" si="16">S20*L20</f>
+        <f t="shared" ref="S37:S42" si="19">S20*L20</f>
         <v>0</v>
       </c>
       <c r="T37" s="50"/>
@@ -6048,7 +6048,7 @@
       <c r="X37" s="3"/>
       <c r="Y37" s="102"/>
       <c r="Z37" s="168">
-        <f t="shared" ref="Z37:Z42" si="17">Z20*L20</f>
+        <f t="shared" ref="Z37:Z42" si="20">Z20*L20</f>
         <v>0</v>
       </c>
       <c r="AA37" s="50"/>
@@ -6058,7 +6058,7 @@
       <c r="AE37" s="3"/>
       <c r="AF37" s="102"/>
       <c r="AG37" s="168">
-        <f t="shared" ref="AG37:AG42" si="18">AG20*L20</f>
+        <f t="shared" ref="AG37:AG42" si="21">AG20*L20</f>
         <v>0</v>
       </c>
       <c r="AH37" s="50"/>
@@ -6069,7 +6069,7 @@
       <c r="AM37" s="102"/>
       <c r="AN37" s="102"/>
       <c r="AO37" s="168">
-        <f t="shared" ref="AO37:AO42" si="19">AO20*L20</f>
+        <f t="shared" ref="AO37:AO42" si="22">AO20*L20</f>
         <v>0</v>
       </c>
       <c r="AP37" s="50"/>
@@ -6080,13 +6080,13 @@
       <c r="AU37" s="102"/>
       <c r="AV37" s="102"/>
       <c r="AW37" s="168">
-        <f t="shared" ref="AW37:AW42" si="20">AW20*L20</f>
+        <f t="shared" ref="AW37:AW42" si="23">AW20*L20</f>
         <v>0</v>
       </c>
       <c r="AX37" s="50"/>
       <c r="AY37" s="53"/>
       <c r="AZ37" s="168">
-        <f>SUM(S37+Z37+AG37+AO37+AW37)</f>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="BA37" s="17"/>
@@ -6121,7 +6121,7 @@
       <c r="Q38" s="3"/>
       <c r="R38" s="3"/>
       <c r="S38" s="168">
-        <f t="shared" si="16"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="T38" s="50"/>
@@ -6131,7 +6131,7 @@
       <c r="X38" s="3"/>
       <c r="Y38" s="102"/>
       <c r="Z38" s="168">
-        <f t="shared" si="17"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="AA38" s="50"/>
@@ -6141,7 +6141,7 @@
       <c r="AE38" s="3"/>
       <c r="AF38" s="102"/>
       <c r="AG38" s="168">
-        <f t="shared" si="18"/>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="AH38" s="50"/>
@@ -6152,7 +6152,7 @@
       <c r="AM38" s="102"/>
       <c r="AN38" s="102"/>
       <c r="AO38" s="168">
-        <f t="shared" si="19"/>
+        <f t="shared" si="22"/>
         <v>0</v>
       </c>
       <c r="AP38" s="50"/>
@@ -6163,13 +6163,13 @@
       <c r="AU38" s="102"/>
       <c r="AV38" s="102"/>
       <c r="AW38" s="168">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="AX38" s="50"/>
       <c r="AY38" s="53"/>
       <c r="AZ38" s="168">
-        <f>SUM(S38+Z38+AG38+AO38+AW38)</f>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="BA38" s="17"/>
@@ -6205,7 +6205,7 @@
       <c r="R39" s="3"/>
       <c r="S39" s="168">
         <f>(S22*L22)+('GRA Insurance'!A2*Q22)</f>
-        <v>9912.9599999999991</v>
+        <v>10512.96</v>
       </c>
       <c r="T39" s="50"/>
       <c r="U39" s="101"/>
@@ -6215,7 +6215,7 @@
       <c r="Y39" s="102"/>
       <c r="Z39" s="168">
         <f>(Z22*L22)+('GRA Insurance'!B2*X22)</f>
-        <v>10276.608</v>
+        <v>10894.608</v>
       </c>
       <c r="AA39" s="50"/>
       <c r="AB39" s="101"/>
@@ -6252,8 +6252,8 @@
       <c r="AX39" s="50"/>
       <c r="AY39" s="53"/>
       <c r="AZ39" s="168">
-        <f>SUM(S39+Z39+AG39+AO39+AW39)</f>
-        <v>20189.567999999999</v>
+        <f t="shared" si="18"/>
+        <v>21407.567999999999</v>
       </c>
       <c r="BA39" s="17"/>
       <c r="BB39" s="21"/>
@@ -6287,7 +6287,7 @@
       <c r="Q40" s="3"/>
       <c r="R40" s="3"/>
       <c r="S40" s="168">
-        <f t="shared" si="16"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="T40" s="50"/>
@@ -6297,7 +6297,7 @@
       <c r="X40" s="3"/>
       <c r="Y40" s="102"/>
       <c r="Z40" s="168">
-        <f t="shared" si="17"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="AA40" s="50"/>
@@ -6307,7 +6307,7 @@
       <c r="AE40" s="3"/>
       <c r="AF40" s="102"/>
       <c r="AG40" s="168">
-        <f t="shared" si="18"/>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="AH40" s="50"/>
@@ -6318,7 +6318,7 @@
       <c r="AM40" s="102"/>
       <c r="AN40" s="102"/>
       <c r="AO40" s="168">
-        <f t="shared" si="19"/>
+        <f t="shared" si="22"/>
         <v>0</v>
       </c>
       <c r="AP40" s="50"/>
@@ -6329,13 +6329,13 @@
       <c r="AU40" s="102"/>
       <c r="AV40" s="102"/>
       <c r="AW40" s="168">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="AX40" s="50"/>
       <c r="AY40" s="53"/>
       <c r="AZ40" s="168">
-        <f>SUM(S40+Z40+AG40+AO40+AW40)</f>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="BA40" s="17"/>
@@ -6370,7 +6370,7 @@
       <c r="Q41" s="3"/>
       <c r="R41" s="3"/>
       <c r="S41" s="168">
-        <f t="shared" si="16"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="T41" s="50"/>
@@ -6380,7 +6380,7 @@
       <c r="X41" s="3"/>
       <c r="Y41" s="102"/>
       <c r="Z41" s="168">
-        <f t="shared" si="17"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="AA41" s="50"/>
@@ -6390,7 +6390,7 @@
       <c r="AE41" s="3"/>
       <c r="AF41" s="102"/>
       <c r="AG41" s="168">
-        <f t="shared" si="18"/>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="AH41" s="50"/>
@@ -6401,7 +6401,7 @@
       <c r="AM41" s="102"/>
       <c r="AN41" s="102"/>
       <c r="AO41" s="168">
-        <f t="shared" si="19"/>
+        <f t="shared" si="22"/>
         <v>0</v>
       </c>
       <c r="AP41" s="50"/>
@@ -6412,13 +6412,13 @@
       <c r="AU41" s="102"/>
       <c r="AV41" s="102"/>
       <c r="AW41" s="168">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="AX41" s="50"/>
       <c r="AY41" s="53"/>
       <c r="AZ41" s="168">
-        <f>SUM(S41+Z41+AG41+AO41+AW41)</f>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="BA41" s="17"/>
@@ -6453,7 +6453,7 @@
       <c r="Q42" s="3"/>
       <c r="R42" s="3"/>
       <c r="S42" s="169">
-        <f t="shared" si="16"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="T42" s="50"/>
@@ -6463,7 +6463,7 @@
       <c r="X42" s="3"/>
       <c r="Y42" s="102"/>
       <c r="Z42" s="169">
-        <f t="shared" si="17"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="AA42" s="50"/>
@@ -6473,7 +6473,7 @@
       <c r="AE42" s="3"/>
       <c r="AF42" s="102"/>
       <c r="AG42" s="169">
-        <f t="shared" si="18"/>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="AH42" s="50"/>
@@ -6484,7 +6484,7 @@
       <c r="AM42" s="102"/>
       <c r="AN42" s="102"/>
       <c r="AO42" s="169">
-        <f t="shared" si="19"/>
+        <f t="shared" si="22"/>
         <v>0</v>
       </c>
       <c r="AP42" s="50"/>
@@ -6495,13 +6495,13 @@
       <c r="AU42" s="102"/>
       <c r="AV42" s="102"/>
       <c r="AW42" s="169">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="AX42" s="50"/>
       <c r="AY42" s="53"/>
       <c r="AZ42" s="169">
-        <f>SUM(S42+Z42+AG42+AO42+AW42)</f>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="BA42" s="17"/>
@@ -6535,7 +6535,7 @@
       <c r="R43" s="3"/>
       <c r="S43" s="167">
         <f>SUM(S31:S42)</f>
-        <v>13661.084799999999</v>
+        <v>14261.084799999999</v>
       </c>
       <c r="T43" s="70"/>
       <c r="U43" s="101"/>
@@ -6545,7 +6545,7 @@
       <c r="Y43" s="102"/>
       <c r="Z43" s="167">
         <f>SUM(Z31:Z42)</f>
-        <v>14137.176544</v>
+        <v>14755.176544</v>
       </c>
       <c r="AA43" s="70"/>
       <c r="AB43" s="71"/>
@@ -6583,7 +6583,7 @@
       <c r="AY43" s="74"/>
       <c r="AZ43" s="167">
         <f>SUM(AZ31:AZ42)</f>
-        <v>27798.261343999999</v>
+        <v>29016.261343999999</v>
       </c>
       <c r="BA43" s="17"/>
       <c r="BB43" s="21"/>
@@ -6677,7 +6677,7 @@
       <c r="R45" s="95"/>
       <c r="S45" s="172">
         <f>SUM(S28+S43)</f>
-        <v>51773.974799999996</v>
+        <v>54773.974799999996</v>
       </c>
       <c r="T45" s="106"/>
       <c r="U45" s="107"/>
@@ -6690,7 +6690,7 @@
       </c>
       <c r="Z45" s="172">
         <f>SUM(Z28+Z43)</f>
-        <v>53393.453244000004</v>
+        <v>56483.453244000004</v>
       </c>
       <c r="AA45" s="106"/>
       <c r="AB45" s="107"/>
@@ -6737,7 +6737,7 @@
       <c r="AY45" s="107"/>
       <c r="AZ45" s="168">
         <f>SUM(S45+Z45+AG45+AO45+AW45)</f>
-        <v>105167.428044</v>
+        <v>111257.428044</v>
       </c>
       <c r="BA45" s="96"/>
       <c r="BB45" s="97"/>
@@ -6812,13 +6812,13 @@
       <c r="A47" s="22" t="s">
         <v>45</v>
       </c>
-      <c r="B47" s="222" t="s">
+      <c r="B47" s="205" t="s">
         <v>111</v>
       </c>
-      <c r="C47" s="216"/>
-      <c r="D47" s="217"/>
-      <c r="E47" s="217"/>
-      <c r="F47" s="218"/>
+      <c r="C47" s="206"/>
+      <c r="D47" s="207"/>
+      <c r="E47" s="207"/>
+      <c r="F47" s="208"/>
       <c r="G47" s="23"/>
       <c r="H47" s="23"/>
       <c r="I47" s="23"/>
@@ -6876,18 +6876,18 @@
     <row r="48" spans="1:59" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2"/>
       <c r="B48" s="3"/>
-      <c r="C48" s="230" t="s">
+      <c r="C48" s="209" t="s">
         <v>46</v>
       </c>
-      <c r="D48" s="231"/>
-      <c r="E48" s="231"/>
-      <c r="F48" s="231"/>
-      <c r="G48" s="231"/>
-      <c r="H48" s="231"/>
-      <c r="I48" s="231"/>
-      <c r="J48" s="231"/>
-      <c r="K48" s="231"/>
-      <c r="L48" s="231"/>
+      <c r="D48" s="210"/>
+      <c r="E48" s="210"/>
+      <c r="F48" s="210"/>
+      <c r="G48" s="210"/>
+      <c r="H48" s="210"/>
+      <c r="I48" s="210"/>
+      <c r="J48" s="210"/>
+      <c r="K48" s="210"/>
+      <c r="L48" s="210"/>
       <c r="M48" s="98"/>
       <c r="N48" s="21"/>
       <c r="O48" s="3"/>
@@ -6952,18 +6952,18 @@
     <row r="49" spans="1:59" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2"/>
       <c r="B49" s="3"/>
-      <c r="C49" s="230" t="s">
+      <c r="C49" s="209" t="s">
         <v>47</v>
       </c>
-      <c r="D49" s="231"/>
-      <c r="E49" s="231"/>
-      <c r="F49" s="231"/>
-      <c r="G49" s="231"/>
-      <c r="H49" s="231"/>
-      <c r="I49" s="231"/>
-      <c r="J49" s="231"/>
-      <c r="K49" s="231"/>
-      <c r="L49" s="231"/>
+      <c r="D49" s="210"/>
+      <c r="E49" s="210"/>
+      <c r="F49" s="210"/>
+      <c r="G49" s="210"/>
+      <c r="H49" s="210"/>
+      <c r="I49" s="210"/>
+      <c r="J49" s="210"/>
+      <c r="K49" s="210"/>
+      <c r="L49" s="210"/>
       <c r="M49" s="98"/>
       <c r="N49" s="21"/>
       <c r="O49" s="3"/>
@@ -7028,18 +7028,18 @@
     <row r="50" spans="1:59" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2"/>
       <c r="B50" s="3"/>
-      <c r="C50" s="230" t="s">
+      <c r="C50" s="209" t="s">
         <v>48</v>
       </c>
-      <c r="D50" s="231"/>
-      <c r="E50" s="231"/>
-      <c r="F50" s="231"/>
-      <c r="G50" s="231"/>
-      <c r="H50" s="231"/>
-      <c r="I50" s="231"/>
-      <c r="J50" s="231"/>
-      <c r="K50" s="231"/>
-      <c r="L50" s="231"/>
+      <c r="D50" s="210"/>
+      <c r="E50" s="210"/>
+      <c r="F50" s="210"/>
+      <c r="G50" s="210"/>
+      <c r="H50" s="210"/>
+      <c r="I50" s="210"/>
+      <c r="J50" s="210"/>
+      <c r="K50" s="210"/>
+      <c r="L50" s="210"/>
       <c r="M50" s="98"/>
       <c r="N50" s="21"/>
       <c r="O50" s="3"/>
@@ -7283,7 +7283,7 @@
       <c r="Q53" s="3"/>
       <c r="R53" s="3"/>
       <c r="S53" s="112">
-        <v>2400</v>
+        <v>4435</v>
       </c>
       <c r="T53" s="50"/>
       <c r="U53" s="116"/>
@@ -7292,7 +7292,7 @@
       <c r="X53" s="3"/>
       <c r="Y53" s="117"/>
       <c r="Z53" s="112">
-        <v>2400</v>
+        <v>4435</v>
       </c>
       <c r="AA53" s="50"/>
       <c r="AB53" s="116"/>
@@ -7327,7 +7327,7 @@
       <c r="AY53" s="53"/>
       <c r="AZ53" s="168">
         <f>SUM(S53+Z53+AG53+AO53+AW53)</f>
-        <v>4800</v>
+        <v>8870</v>
       </c>
       <c r="BA53" s="17"/>
       <c r="BB53" s="21"/>
@@ -7438,7 +7438,7 @@
       <c r="R55" s="3"/>
       <c r="S55" s="167">
         <f>SUM(S53:S54)</f>
-        <v>2400</v>
+        <v>4435</v>
       </c>
       <c r="T55" s="70"/>
       <c r="U55" s="118"/>
@@ -7448,7 +7448,7 @@
       <c r="Y55" s="119"/>
       <c r="Z55" s="167">
         <f>SUM(Z53:Z54)</f>
-        <v>2400</v>
+        <v>4435</v>
       </c>
       <c r="AA55" s="70"/>
       <c r="AB55" s="118"/>
@@ -7486,7 +7486,7 @@
       <c r="AY55" s="74"/>
       <c r="AZ55" s="167">
         <f>SUM(AZ53:AZ54)</f>
-        <v>4800</v>
+        <v>8870</v>
       </c>
       <c r="BA55" s="17"/>
       <c r="BB55" s="21"/>
@@ -8262,7 +8262,8 @@
       <c r="X66" s="95"/>
       <c r="Y66" s="115"/>
       <c r="Z66" s="112">
-        <v>1900</v>
+        <f>1900 * 3</f>
+        <v>5700</v>
       </c>
       <c r="AA66" s="50"/>
       <c r="AB66" s="53"/>
@@ -8297,7 +8298,7 @@
       <c r="AY66" s="74"/>
       <c r="AZ66" s="168">
         <f>SUM(S66+Z66+AG66+AO66+AW66)</f>
-        <v>3800</v>
+        <v>7600</v>
       </c>
       <c r="BA66" s="17"/>
       <c r="BB66" s="21"/>
@@ -8534,17 +8535,17 @@
       <c r="C70" s="120" t="s">
         <v>66</v>
       </c>
-      <c r="D70" s="232" t="s">
+      <c r="D70" s="211" t="s">
         <v>88</v>
       </c>
-      <c r="E70" s="233"/>
-      <c r="F70" s="233"/>
-      <c r="G70" s="233"/>
-      <c r="H70" s="233"/>
-      <c r="I70" s="233"/>
-      <c r="J70" s="233"/>
-      <c r="K70" s="233"/>
-      <c r="L70" s="233"/>
+      <c r="E70" s="212"/>
+      <c r="F70" s="212"/>
+      <c r="G70" s="212"/>
+      <c r="H70" s="212"/>
+      <c r="I70" s="212"/>
+      <c r="J70" s="212"/>
+      <c r="K70" s="212"/>
+      <c r="L70" s="212"/>
       <c r="M70" s="17"/>
       <c r="N70" s="21"/>
       <c r="O70" s="95"/>
@@ -8595,7 +8596,7 @@
       <c r="AX70" s="70"/>
       <c r="AY70" s="74"/>
       <c r="AZ70" s="168">
-        <f>SUM(S70+Z70+AG70+AO70+AW70)</f>
+        <f t="shared" ref="AZ70:AZ75" si="24">SUM(S70+Z70+AG70+AO70+AW70)</f>
         <v>0</v>
       </c>
       <c r="BA70" s="17"/>
@@ -8612,17 +8613,17 @@
       <c r="C71" s="120" t="s">
         <v>67</v>
       </c>
-      <c r="D71" s="232" t="s">
+      <c r="D71" s="211" t="s">
         <v>89</v>
       </c>
-      <c r="E71" s="233"/>
-      <c r="F71" s="233"/>
-      <c r="G71" s="233"/>
-      <c r="H71" s="233"/>
-      <c r="I71" s="233"/>
-      <c r="J71" s="233"/>
-      <c r="K71" s="233"/>
-      <c r="L71" s="233"/>
+      <c r="E71" s="212"/>
+      <c r="F71" s="212"/>
+      <c r="G71" s="212"/>
+      <c r="H71" s="212"/>
+      <c r="I71" s="212"/>
+      <c r="J71" s="212"/>
+      <c r="K71" s="212"/>
+      <c r="L71" s="212"/>
       <c r="M71" s="17"/>
       <c r="N71" s="21"/>
       <c r="O71" s="95"/>
@@ -8673,7 +8674,7 @@
       <c r="AX71" s="70"/>
       <c r="AY71" s="74"/>
       <c r="AZ71" s="168">
-        <f>SUM(S71+Z71+AG71+AO71+AW71)</f>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
       <c r="BA71" s="17"/>
@@ -8690,17 +8691,17 @@
       <c r="C72" s="120" t="s">
         <v>68</v>
       </c>
-      <c r="D72" s="232" t="s">
+      <c r="D72" s="211" t="s">
         <v>90</v>
       </c>
-      <c r="E72" s="232"/>
-      <c r="F72" s="232"/>
-      <c r="G72" s="232"/>
-      <c r="H72" s="232"/>
-      <c r="I72" s="232"/>
-      <c r="J72" s="232"/>
-      <c r="K72" s="232"/>
-      <c r="L72" s="232"/>
+      <c r="E72" s="211"/>
+      <c r="F72" s="211"/>
+      <c r="G72" s="211"/>
+      <c r="H72" s="211"/>
+      <c r="I72" s="211"/>
+      <c r="J72" s="211"/>
+      <c r="K72" s="211"/>
+      <c r="L72" s="211"/>
       <c r="M72" s="17"/>
       <c r="N72" s="21"/>
       <c r="O72" s="95"/>
@@ -8751,7 +8752,7 @@
       <c r="AX72" s="70"/>
       <c r="AY72" s="74"/>
       <c r="AZ72" s="168">
-        <f>SUM(S72+Z72+AG72+AO72+AW72)</f>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
       <c r="BA72" s="17"/>
@@ -8768,17 +8769,17 @@
       <c r="C73" s="120" t="s">
         <v>69</v>
       </c>
-      <c r="D73" s="232" t="s">
+      <c r="D73" s="211" t="s">
         <v>91</v>
       </c>
-      <c r="E73" s="232"/>
-      <c r="F73" s="232"/>
-      <c r="G73" s="232"/>
-      <c r="H73" s="232"/>
-      <c r="I73" s="232"/>
-      <c r="J73" s="232"/>
-      <c r="K73" s="232"/>
-      <c r="L73" s="232"/>
+      <c r="E73" s="211"/>
+      <c r="F73" s="211"/>
+      <c r="G73" s="211"/>
+      <c r="H73" s="211"/>
+      <c r="I73" s="211"/>
+      <c r="J73" s="211"/>
+      <c r="K73" s="211"/>
+      <c r="L73" s="211"/>
       <c r="M73" s="17"/>
       <c r="N73" s="21"/>
       <c r="O73" s="95"/>
@@ -8829,7 +8830,7 @@
       <c r="AX73" s="70"/>
       <c r="AY73" s="74"/>
       <c r="AZ73" s="168">
-        <f>SUM(S73+Z73+AG73+AO73+AW73)</f>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
       <c r="BA73" s="17"/>
@@ -8846,17 +8847,17 @@
       <c r="C74" s="120" t="s">
         <v>103</v>
       </c>
-      <c r="D74" s="232" t="s">
+      <c r="D74" s="211" t="s">
         <v>106</v>
       </c>
-      <c r="E74" s="232"/>
-      <c r="F74" s="232"/>
-      <c r="G74" s="232"/>
-      <c r="H74" s="232"/>
-      <c r="I74" s="232"/>
-      <c r="J74" s="232"/>
-      <c r="K74" s="232"/>
-      <c r="L74" s="232"/>
+      <c r="E74" s="211"/>
+      <c r="F74" s="211"/>
+      <c r="G74" s="211"/>
+      <c r="H74" s="211"/>
+      <c r="I74" s="211"/>
+      <c r="J74" s="211"/>
+      <c r="K74" s="211"/>
+      <c r="L74" s="211"/>
       <c r="M74" s="17"/>
       <c r="N74" s="21"/>
       <c r="O74" s="95"/>
@@ -8907,7 +8908,7 @@
       <c r="AX74" s="70"/>
       <c r="AY74" s="74"/>
       <c r="AZ74" s="168">
-        <f>SUM(S74+Z74+AG74+AO74+AW74)</f>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
       <c r="BA74" s="17"/>
@@ -8924,17 +8925,17 @@
       <c r="C75" s="120" t="s">
         <v>104</v>
       </c>
-      <c r="D75" s="232" t="s">
+      <c r="D75" s="211" t="s">
         <v>105</v>
       </c>
-      <c r="E75" s="232"/>
-      <c r="F75" s="232"/>
-      <c r="G75" s="232"/>
-      <c r="H75" s="232"/>
-      <c r="I75" s="232"/>
-      <c r="J75" s="232"/>
-      <c r="K75" s="232"/>
-      <c r="L75" s="232"/>
+      <c r="E75" s="211"/>
+      <c r="F75" s="211"/>
+      <c r="G75" s="211"/>
+      <c r="H75" s="211"/>
+      <c r="I75" s="211"/>
+      <c r="J75" s="211"/>
+      <c r="K75" s="211"/>
+      <c r="L75" s="211"/>
       <c r="M75" s="17"/>
       <c r="N75" s="21"/>
       <c r="O75" s="95"/>
@@ -8985,7 +8986,7 @@
       <c r="AX75" s="70"/>
       <c r="AY75" s="74"/>
       <c r="AZ75" s="168">
-        <f>SUM(S75+Z75+AG75+AO75+AW75)</f>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
       <c r="BA75" s="17"/>
@@ -9221,15 +9222,15 @@
       <c r="C79" s="161" t="s">
         <v>71</v>
       </c>
-      <c r="D79" s="228"/>
-      <c r="E79" s="229"/>
-      <c r="F79" s="229"/>
-      <c r="G79" s="229"/>
-      <c r="H79" s="229"/>
-      <c r="I79" s="229"/>
-      <c r="J79" s="229"/>
-      <c r="K79" s="229"/>
-      <c r="L79" s="229"/>
+      <c r="D79" s="203"/>
+      <c r="E79" s="204"/>
+      <c r="F79" s="204"/>
+      <c r="G79" s="204"/>
+      <c r="H79" s="204"/>
+      <c r="I79" s="204"/>
+      <c r="J79" s="204"/>
+      <c r="K79" s="204"/>
+      <c r="L79" s="204"/>
       <c r="M79" s="17"/>
       <c r="N79" s="21"/>
       <c r="O79" s="95"/>
@@ -9299,15 +9300,15 @@
       <c r="C80" s="161" t="s">
         <v>71</v>
       </c>
-      <c r="D80" s="228"/>
-      <c r="E80" s="229"/>
-      <c r="F80" s="229"/>
-      <c r="G80" s="229"/>
-      <c r="H80" s="229"/>
-      <c r="I80" s="229"/>
-      <c r="J80" s="229"/>
-      <c r="K80" s="229"/>
-      <c r="L80" s="229"/>
+      <c r="D80" s="203"/>
+      <c r="E80" s="204"/>
+      <c r="F80" s="204"/>
+      <c r="G80" s="204"/>
+      <c r="H80" s="204"/>
+      <c r="I80" s="204"/>
+      <c r="J80" s="204"/>
+      <c r="K80" s="204"/>
+      <c r="L80" s="204"/>
       <c r="M80" s="17"/>
       <c r="N80" s="21"/>
       <c r="O80" s="95"/>
@@ -9402,7 +9403,7 @@
       <c r="Y81" s="80"/>
       <c r="Z81" s="167">
         <f>SUM(Z65:Z80)</f>
-        <v>1900</v>
+        <v>5700</v>
       </c>
       <c r="AA81" s="70"/>
       <c r="AB81" s="74"/>
@@ -9440,7 +9441,7 @@
       <c r="AY81" s="74"/>
       <c r="AZ81" s="167">
         <f>SUM(AZ65:AZ80)</f>
-        <v>3800</v>
+        <v>7600</v>
       </c>
       <c r="BA81" s="17"/>
       <c r="BB81" s="21"/>
@@ -9536,7 +9537,7 @@
       <c r="R83" s="131"/>
       <c r="S83" s="168">
         <f>SUM(S45+S51+S55+S62+S81)</f>
-        <v>56073.974799999996</v>
+        <v>61108.974799999996</v>
       </c>
       <c r="T83" s="50"/>
       <c r="U83" s="79"/>
@@ -9546,7 +9547,7 @@
       <c r="Y83" s="77"/>
       <c r="Z83" s="168">
         <f>SUM(Z45+Z51+Z55+Z62+Z81)</f>
-        <v>57693.453244000004</v>
+        <v>66618.453244000004</v>
       </c>
       <c r="AA83" s="50"/>
       <c r="AB83" s="79"/>
@@ -9584,7 +9585,7 @@
       <c r="AY83" s="53"/>
       <c r="AZ83" s="168">
         <f>SUM(S83+Z83+AG83+AO83+AW83)</f>
-        <v>113767.428044</v>
+        <v>127727.428044</v>
       </c>
       <c r="BA83" s="17"/>
       <c r="BB83" s="21"/>
@@ -9745,7 +9746,7 @@
       <c r="R86" s="95"/>
       <c r="S86" s="168">
         <f>IF($L86&gt;0,SUM(S83-S77-S51-OR($L$58="Yes",ISBLANK($L$58))*S58-OR($L$59="Yes",ISBLANK($L$59))*S59-OR($L$60="Yes",ISBLANK($L$60))*S60-OR($L$61="Yes",ISBLANK($L$61))*S61-S105,0),0)</f>
-        <v>56073.974799999996</v>
+        <v>61108.974799999996</v>
       </c>
       <c r="T86" s="70"/>
       <c r="U86" s="74"/>
@@ -9755,7 +9756,7 @@
       <c r="Y86" s="80"/>
       <c r="Z86" s="168">
         <f>IF($L86&gt;0,SUM(Z83-Z77-Z51-OR($L$58="yes",ISBLANK($L$58))*Z58-OR($L$59="yes",ISBLANK($L$59))*Z59-OR($L$60="yes",ISBLANK($L$60))*Z60-OR($L$61="yes",ISBLANK($L$61))*Z61-Z105,0),0)</f>
-        <v>57693.453244000004</v>
+        <v>66618.453244000004</v>
       </c>
       <c r="AA86" s="70"/>
       <c r="AB86" s="138"/>
@@ -9793,7 +9794,7 @@
       <c r="AY86" s="53"/>
       <c r="AZ86" s="168">
         <f>SUM(S86+Z86+AG86+AO86+AW86)</f>
-        <v>113767.428044</v>
+        <v>127727.428044</v>
       </c>
       <c r="BA86" s="17"/>
       <c r="BB86" s="21"/>
@@ -9909,7 +9910,7 @@
       <c r="R88" s="95"/>
       <c r="S88" s="169">
         <f>S86*$L86+S87</f>
-        <v>31401.425888000002</v>
+        <v>34221.025888000004</v>
       </c>
       <c r="T88" s="50"/>
       <c r="U88" s="53"/>
@@ -9919,7 +9920,7 @@
       <c r="Y88" s="115"/>
       <c r="Z88" s="169">
         <f>Z86*$L86+Z87</f>
-        <v>32308.333816640006</v>
+        <v>37306.333816640006</v>
       </c>
       <c r="AA88" s="50"/>
       <c r="AB88" s="79"/>
@@ -9957,7 +9958,7 @@
       <c r="AY88" s="53"/>
       <c r="AZ88" s="169">
         <f>SUM(S88+Z88+AG88+AO88+AW88)</f>
-        <v>63709.759704640004</v>
+        <v>71527.35970464001</v>
       </c>
       <c r="BA88" s="17"/>
       <c r="BB88" s="21"/>
@@ -10073,7 +10074,7 @@
       <c r="R90" s="9"/>
       <c r="S90" s="174">
         <f>SUM(S83+S88)</f>
-        <v>87475.400687999994</v>
+        <v>95330.000688</v>
       </c>
       <c r="T90" s="143"/>
       <c r="U90" s="144"/>
@@ -10083,7 +10084,7 @@
       <c r="Y90" s="145"/>
       <c r="Z90" s="174">
         <f>SUM(Z83+Z88)</f>
-        <v>90001.78706064001</v>
+        <v>103924.78706064001</v>
       </c>
       <c r="AA90" s="143"/>
       <c r="AB90" s="144"/>
@@ -10121,7 +10122,7 @@
       <c r="AY90" s="146"/>
       <c r="AZ90" s="174">
         <f>SUM(AZ83+AZ88)</f>
-        <v>177477.18774864002</v>
+        <v>199254.78774864</v>
       </c>
       <c r="BA90" s="96"/>
       <c r="BB90" s="97"/>
@@ -11099,6 +11100,29 @@
     </row>
   </sheetData>
   <mergeCells count="39">
+    <mergeCell ref="E4:K4"/>
+    <mergeCell ref="E2:K2"/>
+    <mergeCell ref="U2:AG2"/>
+    <mergeCell ref="V7:Z7"/>
+    <mergeCell ref="AC7:AG7"/>
+    <mergeCell ref="AM7:AO7"/>
+    <mergeCell ref="AU7:AW7"/>
+    <mergeCell ref="V4:X4"/>
+    <mergeCell ref="AU4:AW4"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="B30:F30"/>
+    <mergeCell ref="Q7:S7"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="C9:F9"/>
+    <mergeCell ref="O9:O10"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="AS9:AS10"/>
+    <mergeCell ref="AZ9:AZ10"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="AK9:AK10"/>
+    <mergeCell ref="C15:D15"/>
     <mergeCell ref="AA4:AC4"/>
     <mergeCell ref="AE4:AG4"/>
     <mergeCell ref="D79:L79"/>
@@ -11115,29 +11139,6 @@
     <mergeCell ref="D75:L75"/>
     <mergeCell ref="V9:V10"/>
     <mergeCell ref="AC9:AC10"/>
-    <mergeCell ref="AS9:AS10"/>
-    <mergeCell ref="AZ9:AZ10"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="AK9:AK10"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="B19:D19"/>
-    <mergeCell ref="B30:F30"/>
-    <mergeCell ref="Q7:S7"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="C9:F9"/>
-    <mergeCell ref="O9:O10"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="V7:Z7"/>
-    <mergeCell ref="AC7:AG7"/>
-    <mergeCell ref="AM7:AO7"/>
-    <mergeCell ref="AU7:AW7"/>
-    <mergeCell ref="V4:X4"/>
-    <mergeCell ref="AU4:AW4"/>
-    <mergeCell ref="E4:K4"/>
-    <mergeCell ref="E2:K2"/>
-    <mergeCell ref="U2:AG2"/>
   </mergeCells>
   <conditionalFormatting sqref="AM18:AQ18 AU18:AY18 S18:V19 Y18:AC19 AF18:AI19 AK19 AN19:AQ19 AS19 AV19:AY19 T20:U25 Y20:Y25 AA20:AB25 AF20:AF25 AH20:AI25 AN20:AN25 AP20:AQ25 AV20:AV25 AX20:AY25 S26:V29 Y26:AC29 AF26:AI29 AM26:AQ29 AU26:AY29 U52:V57 Y52:Y57 AB52:AC57 AF52:AF57 AI52:AI57 AM52:AN57 AQ52:AQ57 AU52:AV57 U83:V85 Y83:Y85 AI83:AI86 AM83:AN86 AQ83:AQ86 AU83:AV86 U90:V90 Y90 AB83:AC90 AF83:AF90 AI88:AI90 AM88:AN90 AQ88:AQ90 AU88:AV90 S91:V91 Y91:AC91 AF91:AI91 AM91:AQ91 AU91:AX91 AI92">
     <cfRule type="cellIs" dxfId="0" priority="1" stopIfTrue="1" operator="lessThan">
@@ -11297,39 +11298,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A1" s="240" t="s">
+      <c r="A1" s="244" t="s">
         <v>131</v>
       </c>
-      <c r="B1" s="240" t="s">
+      <c r="B1" s="244" t="s">
         <v>145</v>
       </c>
-      <c r="C1" s="240" t="s">
+      <c r="C1" s="244" t="s">
         <v>133</v>
       </c>
-      <c r="D1" s="242"/>
-      <c r="E1" s="240" t="s">
+      <c r="D1" s="246"/>
+      <c r="E1" s="244" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="195" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="241"/>
-      <c r="B2" s="241"/>
+      <c r="A2" s="245"/>
+      <c r="B2" s="245"/>
       <c r="C2" s="184" t="s">
         <v>146</v>
       </c>
       <c r="D2" s="184" t="s">
         <v>150</v>
       </c>
-      <c r="E2" s="241"/>
+      <c r="E2" s="245"/>
     </row>
     <row r="3" spans="1:5" s="195" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="243" t="s">
+      <c r="A3" s="247" t="s">
         <v>132</v>
       </c>
-      <c r="B3" s="244"/>
-      <c r="C3" s="244"/>
-      <c r="D3" s="244"/>
-      <c r="E3" s="245"/>
+      <c r="B3" s="248"/>
+      <c r="C3" s="248"/>
+      <c r="D3" s="248"/>
+      <c r="E3" s="249"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="196"/>
@@ -11352,13 +11353,13 @@
       <c r="E5" s="196"/>
     </row>
     <row r="6" spans="1:5" s="195" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="249" t="s">
+      <c r="A6" s="253" t="s">
         <v>137</v>
       </c>
-      <c r="B6" s="250"/>
-      <c r="C6" s="250"/>
-      <c r="D6" s="250"/>
-      <c r="E6" s="251"/>
+      <c r="B6" s="254"/>
+      <c r="C6" s="254"/>
+      <c r="D6" s="254"/>
+      <c r="E6" s="255"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="196"/>
@@ -11446,13 +11447,13 @@
       <c r="E13" s="196"/>
     </row>
     <row r="14" spans="1:5" s="195" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="246" t="s">
+      <c r="A14" s="250" t="s">
         <v>144</v>
       </c>
-      <c r="B14" s="247"/>
-      <c r="C14" s="247"/>
-      <c r="D14" s="247"/>
-      <c r="E14" s="248"/>
+      <c r="B14" s="251"/>
+      <c r="C14" s="251"/>
+      <c r="D14" s="251"/>
+      <c r="E14" s="252"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" s="196"/>
@@ -11480,13 +11481,13 @@
       <c r="E17" s="196"/>
     </row>
     <row r="18" spans="1:5" s="195" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="252" t="s">
+      <c r="A18" s="256" t="s">
         <v>147</v>
       </c>
-      <c r="B18" s="253"/>
-      <c r="C18" s="253"/>
-      <c r="D18" s="253"/>
-      <c r="E18" s="254"/>
+      <c r="B18" s="257"/>
+      <c r="C18" s="257"/>
+      <c r="D18" s="257"/>
+      <c r="E18" s="258"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" s="196"/>
@@ -11514,13 +11515,13 @@
       <c r="E21" s="196"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A22" s="234" t="s">
+      <c r="A22" s="238" t="s">
         <v>148</v>
       </c>
-      <c r="B22" s="235"/>
-      <c r="C22" s="235"/>
-      <c r="D22" s="235"/>
-      <c r="E22" s="236"/>
+      <c r="B22" s="239"/>
+      <c r="C22" s="239"/>
+      <c r="D22" s="239"/>
+      <c r="E22" s="240"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" s="196"/>
@@ -11548,13 +11549,13 @@
       <c r="E25" s="196"/>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A26" s="237" t="s">
+      <c r="A26" s="241" t="s">
         <v>149</v>
       </c>
-      <c r="B26" s="238"/>
-      <c r="C26" s="238"/>
-      <c r="D26" s="238"/>
-      <c r="E26" s="239"/>
+      <c r="B26" s="242"/>
+      <c r="C26" s="242"/>
+      <c r="D26" s="242"/>
+      <c r="E26" s="243"/>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" s="196"/>

</xml_diff>

<commit_message>
ADAP 2023: Prepare budget details for printng to final PDF
</commit_message>
<xml_diff>
--- a/budget/BudgetDetails.xlsx
+++ b/budget/BudgetDetails.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kpenev/projects/git/proposals/TESS_EB_Bayesian_Proposal/budget/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C8E16A1-0861-394D-87AC-EF44119C9C37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AB4EFC5-2338-2644-B861-E7F25A77C00D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="460" windowWidth="33600" windowHeight="20540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1600,29 +1600,91 @@
     <xf numFmtId="164" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="49" fontId="14" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="3" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="5" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="6" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
@@ -1631,68 +1693,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="3" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="5" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="15" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="13" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="13" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -2962,8 +2962,7 @@
     <col min="49" max="49" width="13.5" style="156" hidden="1" customWidth="1"/>
     <col min="50" max="51" width="1.5" style="156" customWidth="1"/>
     <col min="52" max="52" width="13.5" style="156" customWidth="1"/>
-    <col min="53" max="53" width="15.83203125" style="156" customWidth="1"/>
-    <col min="54" max="59" width="15.83203125" style="156" hidden="1" customWidth="1"/>
+    <col min="53" max="59" width="15.83203125" style="156" hidden="1" customWidth="1"/>
     <col min="60" max="256" width="11.5" style="156" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3035,15 +3034,15 @@
       <c r="D2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="235" t="s">
+      <c r="E2" s="201" t="s">
         <v>151</v>
       </c>
-      <c r="F2" s="235"/>
-      <c r="G2" s="235"/>
-      <c r="H2" s="235"/>
-      <c r="I2" s="235"/>
-      <c r="J2" s="235"/>
-      <c r="K2" s="235"/>
+      <c r="F2" s="201"/>
+      <c r="G2" s="201"/>
+      <c r="H2" s="201"/>
+      <c r="I2" s="201"/>
+      <c r="J2" s="201"/>
+      <c r="K2" s="201"/>
       <c r="L2" s="159"/>
       <c r="M2" s="159"/>
       <c r="N2" s="159"/>
@@ -3055,21 +3054,21 @@
       <c r="T2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="U2" s="236" t="s">
+      <c r="U2" s="202" t="s">
         <v>152</v>
       </c>
-      <c r="V2" s="237"/>
-      <c r="W2" s="237"/>
-      <c r="X2" s="237"/>
-      <c r="Y2" s="237"/>
-      <c r="Z2" s="237"/>
-      <c r="AA2" s="237"/>
-      <c r="AB2" s="237"/>
-      <c r="AC2" s="237"/>
-      <c r="AD2" s="237"/>
-      <c r="AE2" s="237"/>
-      <c r="AF2" s="237"/>
-      <c r="AG2" s="237"/>
+      <c r="V2" s="203"/>
+      <c r="W2" s="203"/>
+      <c r="X2" s="203"/>
+      <c r="Y2" s="203"/>
+      <c r="Z2" s="203"/>
+      <c r="AA2" s="203"/>
+      <c r="AB2" s="203"/>
+      <c r="AC2" s="203"/>
+      <c r="AD2" s="203"/>
+      <c r="AE2" s="203"/>
+      <c r="AF2" s="203"/>
+      <c r="AG2" s="203"/>
       <c r="AH2" s="159"/>
       <c r="AJ2" s="159"/>
       <c r="AK2" s="159"/>
@@ -3164,15 +3163,15 @@
       <c r="D4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="235" t="s">
+      <c r="E4" s="201" t="s">
         <v>154</v>
       </c>
-      <c r="F4" s="235"/>
-      <c r="G4" s="235"/>
-      <c r="H4" s="235"/>
-      <c r="I4" s="235"/>
-      <c r="J4" s="235"/>
-      <c r="K4" s="235"/>
+      <c r="F4" s="201"/>
+      <c r="G4" s="201"/>
+      <c r="H4" s="201"/>
+      <c r="I4" s="201"/>
+      <c r="J4" s="201"/>
+      <c r="K4" s="201"/>
       <c r="L4" s="3"/>
       <c r="M4" s="3"/>
       <c r="N4" s="3"/>
@@ -3185,24 +3184,24 @@
         <v>3</v>
       </c>
       <c r="U4" s="3"/>
-      <c r="V4" s="202">
+      <c r="V4" s="208">
         <v>43965</v>
       </c>
-      <c r="W4" s="202"/>
-      <c r="X4" s="202"/>
+      <c r="W4" s="208"/>
+      <c r="X4" s="208"/>
       <c r="Y4" s="3"/>
       <c r="Z4" s="3"/>
-      <c r="AA4" s="201" t="s">
+      <c r="AA4" s="231" t="s">
         <v>155</v>
       </c>
-      <c r="AB4" s="201"/>
-      <c r="AC4" s="201"/>
+      <c r="AB4" s="231"/>
+      <c r="AC4" s="231"/>
       <c r="AD4" s="159"/>
-      <c r="AE4" s="202">
+      <c r="AE4" s="208">
         <v>44694</v>
       </c>
-      <c r="AF4" s="202"/>
-      <c r="AG4" s="202"/>
+      <c r="AF4" s="208"/>
+      <c r="AG4" s="208"/>
       <c r="AH4" s="159"/>
       <c r="AJ4" s="7"/>
       <c r="AK4" s="7"/>
@@ -3212,11 +3211,11 @@
       <c r="AR4" s="159"/>
       <c r="AS4" s="159"/>
       <c r="AT4" s="159"/>
-      <c r="AU4" s="233" t="s">
+      <c r="AU4" s="209" t="s">
         <v>4</v>
       </c>
-      <c r="AV4" s="234"/>
-      <c r="AW4" s="234"/>
+      <c r="AV4" s="210"/>
+      <c r="AW4" s="210"/>
       <c r="AX4" s="159"/>
       <c r="AY4" s="159"/>
       <c r="AZ4" s="159"/>
@@ -3371,49 +3370,49 @@
       <c r="N7" s="14"/>
       <c r="O7" s="14"/>
       <c r="P7" s="14"/>
-      <c r="Q7" s="226" t="s">
+      <c r="Q7" s="204" t="s">
         <v>97</v>
       </c>
-      <c r="R7" s="227"/>
-      <c r="S7" s="227"/>
+      <c r="R7" s="220"/>
+      <c r="S7" s="220"/>
       <c r="T7" s="14"/>
       <c r="U7" s="14"/>
-      <c r="V7" s="226" t="s">
+      <c r="V7" s="204" t="s">
         <v>98</v>
       </c>
-      <c r="W7" s="230"/>
-      <c r="X7" s="230"/>
-      <c r="Y7" s="231"/>
-      <c r="Z7" s="232"/>
+      <c r="W7" s="205"/>
+      <c r="X7" s="205"/>
+      <c r="Y7" s="206"/>
+      <c r="Z7" s="207"/>
       <c r="AA7" s="14"/>
       <c r="AB7" s="14"/>
-      <c r="AC7" s="226" t="s">
+      <c r="AC7" s="204" t="s">
         <v>99</v>
       </c>
-      <c r="AD7" s="230"/>
-      <c r="AE7" s="230"/>
-      <c r="AF7" s="231"/>
-      <c r="AG7" s="232"/>
+      <c r="AD7" s="205"/>
+      <c r="AE7" s="205"/>
+      <c r="AF7" s="206"/>
+      <c r="AG7" s="207"/>
       <c r="AH7" s="14"/>
       <c r="AI7" s="14"/>
       <c r="AJ7" s="14"/>
       <c r="AK7" s="14"/>
       <c r="AL7" s="14"/>
-      <c r="AM7" s="226" t="s">
+      <c r="AM7" s="204" t="s">
         <v>6</v>
       </c>
-      <c r="AN7" s="231"/>
-      <c r="AO7" s="232"/>
+      <c r="AN7" s="206"/>
+      <c r="AO7" s="207"/>
       <c r="AP7" s="14"/>
       <c r="AQ7" s="14"/>
       <c r="AR7" s="14"/>
       <c r="AS7" s="14"/>
       <c r="AT7" s="14"/>
-      <c r="AU7" s="226" t="s">
+      <c r="AU7" s="204" t="s">
         <v>7</v>
       </c>
-      <c r="AV7" s="231"/>
-      <c r="AW7" s="232"/>
+      <c r="AV7" s="206"/>
+      <c r="AW7" s="207"/>
       <c r="AX7" s="14"/>
       <c r="AY7" s="14"/>
       <c r="AZ7" s="15"/>
@@ -3491,12 +3490,12 @@
         <v>8</v>
       </c>
       <c r="B9" s="3"/>
-      <c r="C9" s="205" t="s">
+      <c r="C9" s="223" t="s">
         <v>9</v>
       </c>
-      <c r="D9" s="206"/>
-      <c r="E9" s="207"/>
-      <c r="F9" s="208"/>
+      <c r="D9" s="217"/>
+      <c r="E9" s="218"/>
+      <c r="F9" s="219"/>
       <c r="G9" s="23"/>
       <c r="H9" s="23"/>
       <c r="I9" s="23"/>
@@ -3505,7 +3504,7 @@
       <c r="L9" s="24"/>
       <c r="M9" s="25"/>
       <c r="N9" s="26"/>
-      <c r="O9" s="213" t="s">
+      <c r="O9" s="224" t="s">
         <v>10</v>
       </c>
       <c r="P9" s="3"/>
@@ -3514,7 +3513,7 @@
       <c r="S9" s="3"/>
       <c r="T9" s="27"/>
       <c r="U9" s="28"/>
-      <c r="V9" s="213" t="s">
+      <c r="V9" s="224" t="s">
         <v>10</v>
       </c>
       <c r="W9" s="3"/>
@@ -3523,7 +3522,7 @@
       <c r="Z9" s="3"/>
       <c r="AA9" s="27"/>
       <c r="AB9" s="28"/>
-      <c r="AC9" s="213" t="s">
+      <c r="AC9" s="224" t="s">
         <v>10</v>
       </c>
       <c r="AD9" s="3"/>
@@ -3533,7 +3532,7 @@
       <c r="AH9" s="27"/>
       <c r="AI9" s="28"/>
       <c r="AJ9" s="3"/>
-      <c r="AK9" s="213" t="s">
+      <c r="AK9" s="224" t="s">
         <v>10</v>
       </c>
       <c r="AL9" s="3"/>
@@ -3543,7 +3542,7 @@
       <c r="AP9" s="27"/>
       <c r="AQ9" s="28"/>
       <c r="AR9" s="3"/>
-      <c r="AS9" s="213" t="s">
+      <c r="AS9" s="224" t="s">
         <v>10</v>
       </c>
       <c r="AT9" s="3"/>
@@ -3552,7 +3551,7 @@
       <c r="AW9" s="3"/>
       <c r="AX9" s="27"/>
       <c r="AY9" s="29"/>
-      <c r="AZ9" s="213" t="s">
+      <c r="AZ9" s="224" t="s">
         <v>11</v>
       </c>
       <c r="BA9" s="17"/>
@@ -3588,7 +3587,7 @@
       </c>
       <c r="M10" s="25"/>
       <c r="N10" s="26"/>
-      <c r="O10" s="214"/>
+      <c r="O10" s="225"/>
       <c r="P10" s="33"/>
       <c r="Q10" s="32" t="s">
         <v>17</v>
@@ -3599,7 +3598,7 @@
       </c>
       <c r="T10" s="35"/>
       <c r="U10" s="36"/>
-      <c r="V10" s="214"/>
+      <c r="V10" s="225"/>
       <c r="W10" s="33"/>
       <c r="X10" s="32" t="s">
         <v>17</v>
@@ -3610,7 +3609,7 @@
       </c>
       <c r="AA10" s="35"/>
       <c r="AB10" s="36"/>
-      <c r="AC10" s="214"/>
+      <c r="AC10" s="225"/>
       <c r="AD10" s="33"/>
       <c r="AE10" s="32" t="s">
         <v>17</v>
@@ -3622,7 +3621,7 @@
       <c r="AH10" s="35"/>
       <c r="AI10" s="36"/>
       <c r="AJ10" s="33"/>
-      <c r="AK10" s="214"/>
+      <c r="AK10" s="225"/>
       <c r="AL10" s="33"/>
       <c r="AM10" s="32" t="s">
         <v>17</v>
@@ -3634,7 +3633,7 @@
       <c r="AP10" s="35"/>
       <c r="AQ10" s="36"/>
       <c r="AR10" s="33"/>
-      <c r="AS10" s="214"/>
+      <c r="AS10" s="225"/>
       <c r="AT10" s="33"/>
       <c r="AU10" s="32" t="s">
         <v>17</v>
@@ -3645,7 +3644,7 @@
       </c>
       <c r="AX10" s="35"/>
       <c r="AY10" s="38"/>
-      <c r="AZ10" s="215"/>
+      <c r="AZ10" s="226"/>
       <c r="BA10" s="17"/>
       <c r="BB10" s="21"/>
       <c r="BC10" s="3"/>
@@ -3659,10 +3658,10 @@
       <c r="B11" s="39" t="s">
         <v>19</v>
       </c>
-      <c r="C11" s="216" t="s">
+      <c r="C11" s="227" t="s">
         <v>153</v>
       </c>
-      <c r="D11" s="217"/>
+      <c r="D11" s="228"/>
       <c r="E11" s="40"/>
       <c r="F11" s="41">
         <v>11712.89</v>
@@ -3765,15 +3764,15 @@
       <c r="BF11" s="37"/>
       <c r="BG11" s="16"/>
     </row>
-    <row r="12" spans="1:59" ht="19" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:59" ht="19" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="B12" s="39" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="228" t="s">
+      <c r="C12" s="221" t="s">
         <v>156</v>
       </c>
-      <c r="D12" s="229"/>
+      <c r="D12" s="222"/>
       <c r="E12" s="40"/>
       <c r="F12" s="54">
         <v>0</v>
@@ -3876,15 +3875,15 @@
       <c r="BF12" s="37"/>
       <c r="BG12" s="16"/>
     </row>
-    <row r="13" spans="1:59" ht="19" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:59" ht="19" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
       <c r="B13" s="39" t="s">
         <v>21</v>
       </c>
-      <c r="C13" s="228" t="s">
+      <c r="C13" s="221" t="s">
         <v>107</v>
       </c>
-      <c r="D13" s="229"/>
+      <c r="D13" s="222"/>
       <c r="E13" s="40"/>
       <c r="F13" s="54">
         <v>0</v>
@@ -3987,15 +3986,15 @@
       <c r="BF13" s="37"/>
       <c r="BG13" s="16"/>
     </row>
-    <row r="14" spans="1:59" ht="19" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:59" ht="19" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
       <c r="B14" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="C14" s="228" t="s">
+      <c r="C14" s="221" t="s">
         <v>108</v>
       </c>
-      <c r="D14" s="229"/>
+      <c r="D14" s="222"/>
       <c r="E14" s="40"/>
       <c r="F14" s="54">
         <v>0</v>
@@ -4098,15 +4097,15 @@
       <c r="BF14" s="37"/>
       <c r="BG14" s="16"/>
     </row>
-    <row r="15" spans="1:59" ht="19" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:59" ht="19" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
       <c r="B15" s="39" t="s">
         <v>23</v>
       </c>
-      <c r="C15" s="218" t="s">
+      <c r="C15" s="229" t="s">
         <v>109</v>
       </c>
-      <c r="D15" s="219"/>
+      <c r="D15" s="230"/>
       <c r="E15" s="40"/>
       <c r="F15" s="54">
         <v>0</v>
@@ -4209,15 +4208,15 @@
       <c r="BF15" s="37"/>
       <c r="BG15" s="16"/>
     </row>
-    <row r="16" spans="1:59" ht="19" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:59" ht="19" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
       <c r="B16" s="39" t="s">
         <v>24</v>
       </c>
-      <c r="C16" s="220" t="s">
+      <c r="C16" s="211" t="s">
         <v>36</v>
       </c>
-      <c r="D16" s="221"/>
+      <c r="D16" s="212"/>
       <c r="E16" s="40"/>
       <c r="F16" s="59">
         <v>0</v>
@@ -4466,11 +4465,11 @@
       <c r="A19" s="81" t="s">
         <v>26</v>
       </c>
-      <c r="B19" s="222" t="s">
+      <c r="B19" s="213" t="s">
         <v>27</v>
       </c>
-      <c r="C19" s="223"/>
-      <c r="D19" s="224"/>
+      <c r="C19" s="214"/>
+      <c r="D19" s="215"/>
       <c r="E19" s="3"/>
       <c r="F19" s="32" t="s">
         <v>13</v>
@@ -4947,7 +4946,7 @@
       <c r="BF23" s="37"/>
       <c r="BG23" s="6"/>
     </row>
-    <row r="24" spans="1:59" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:59" ht="19" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="2"/>
       <c r="B24" s="39" t="s">
         <v>23</v>
@@ -5048,7 +5047,7 @@
       <c r="BF24" s="37"/>
       <c r="BG24" s="6"/>
     </row>
-    <row r="25" spans="1:59" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:59" ht="19" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="2"/>
       <c r="B25" s="39" t="s">
         <v>24</v>
@@ -5437,13 +5436,13 @@
       <c r="A30" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="B30" s="225" t="s">
+      <c r="B30" s="216" t="s">
         <v>35</v>
       </c>
-      <c r="C30" s="206"/>
-      <c r="D30" s="207"/>
-      <c r="E30" s="207"/>
-      <c r="F30" s="208"/>
+      <c r="C30" s="217"/>
+      <c r="D30" s="218"/>
+      <c r="E30" s="218"/>
+      <c r="F30" s="219"/>
       <c r="G30" s="23"/>
       <c r="H30" s="23"/>
       <c r="I30" s="23"/>
@@ -5584,7 +5583,7 @@
       <c r="BF31" s="5"/>
       <c r="BG31" s="6"/>
     </row>
-    <row r="32" spans="1:59" ht="19" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:59" ht="19" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2"/>
       <c r="B32" s="76" t="s">
         <v>20</v>
@@ -5670,7 +5669,7 @@
       <c r="BF32" s="5"/>
       <c r="BG32" s="6"/>
     </row>
-    <row r="33" spans="1:59" ht="19" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:59" ht="19" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2"/>
       <c r="B33" s="76" t="s">
         <v>21</v>
@@ -5756,7 +5755,7 @@
       <c r="BF33" s="5"/>
       <c r="BG33" s="6"/>
     </row>
-    <row r="34" spans="1:59" ht="19" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:59" ht="19" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2"/>
       <c r="B34" s="76" t="s">
         <v>37</v>
@@ -5842,7 +5841,7 @@
       <c r="BF34" s="5"/>
       <c r="BG34" s="6"/>
     </row>
-    <row r="35" spans="1:59" ht="19" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:59" ht="19" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2"/>
       <c r="B35" s="76" t="s">
         <v>38</v>
@@ -5928,7 +5927,7 @@
       <c r="BF35" s="5"/>
       <c r="BG35" s="6"/>
     </row>
-    <row r="36" spans="1:59" ht="19" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:59" ht="19" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2"/>
       <c r="B36" s="76" t="s">
         <v>24</v>
@@ -6346,7 +6345,7 @@
       <c r="BF40" s="5"/>
       <c r="BG40" s="6"/>
     </row>
-    <row r="41" spans="1:59" ht="19" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:59" ht="19" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2"/>
       <c r="B41" s="76" t="s">
         <v>23</v>
@@ -6429,7 +6428,7 @@
       <c r="BF41" s="5"/>
       <c r="BG41" s="6"/>
     </row>
-    <row r="42" spans="1:59" ht="19" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:59" ht="19" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2"/>
       <c r="B42" s="76" t="s">
         <v>24</v>
@@ -6812,13 +6811,13 @@
       <c r="A47" s="22" t="s">
         <v>45</v>
       </c>
-      <c r="B47" s="205" t="s">
+      <c r="B47" s="223" t="s">
         <v>111</v>
       </c>
-      <c r="C47" s="206"/>
-      <c r="D47" s="207"/>
-      <c r="E47" s="207"/>
-      <c r="F47" s="208"/>
+      <c r="C47" s="217"/>
+      <c r="D47" s="218"/>
+      <c r="E47" s="218"/>
+      <c r="F47" s="219"/>
       <c r="G47" s="23"/>
       <c r="H47" s="23"/>
       <c r="I47" s="23"/>
@@ -6873,21 +6872,21 @@
       <c r="BF47" s="5"/>
       <c r="BG47" s="6"/>
     </row>
-    <row r="48" spans="1:59" ht="19" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:59" ht="19" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2"/>
       <c r="B48" s="3"/>
-      <c r="C48" s="209" t="s">
+      <c r="C48" s="234" t="s">
         <v>46</v>
       </c>
-      <c r="D48" s="210"/>
-      <c r="E48" s="210"/>
-      <c r="F48" s="210"/>
-      <c r="G48" s="210"/>
-      <c r="H48" s="210"/>
-      <c r="I48" s="210"/>
-      <c r="J48" s="210"/>
-      <c r="K48" s="210"/>
-      <c r="L48" s="210"/>
+      <c r="D48" s="235"/>
+      <c r="E48" s="235"/>
+      <c r="F48" s="235"/>
+      <c r="G48" s="235"/>
+      <c r="H48" s="235"/>
+      <c r="I48" s="235"/>
+      <c r="J48" s="235"/>
+      <c r="K48" s="235"/>
+      <c r="L48" s="235"/>
       <c r="M48" s="98"/>
       <c r="N48" s="21"/>
       <c r="O48" s="3"/>
@@ -6949,21 +6948,21 @@
       <c r="BF48" s="5"/>
       <c r="BG48" s="6"/>
     </row>
-    <row r="49" spans="1:59" ht="19" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:59" ht="19" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2"/>
       <c r="B49" s="3"/>
-      <c r="C49" s="209" t="s">
+      <c r="C49" s="234" t="s">
         <v>47</v>
       </c>
-      <c r="D49" s="210"/>
-      <c r="E49" s="210"/>
-      <c r="F49" s="210"/>
-      <c r="G49" s="210"/>
-      <c r="H49" s="210"/>
-      <c r="I49" s="210"/>
-      <c r="J49" s="210"/>
-      <c r="K49" s="210"/>
-      <c r="L49" s="210"/>
+      <c r="D49" s="235"/>
+      <c r="E49" s="235"/>
+      <c r="F49" s="235"/>
+      <c r="G49" s="235"/>
+      <c r="H49" s="235"/>
+      <c r="I49" s="235"/>
+      <c r="J49" s="235"/>
+      <c r="K49" s="235"/>
+      <c r="L49" s="235"/>
       <c r="M49" s="98"/>
       <c r="N49" s="21"/>
       <c r="O49" s="3"/>
@@ -7025,21 +7024,21 @@
       <c r="BF49" s="5"/>
       <c r="BG49" s="6"/>
     </row>
-    <row r="50" spans="1:59" ht="19" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:59" ht="19" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2"/>
       <c r="B50" s="3"/>
-      <c r="C50" s="209" t="s">
+      <c r="C50" s="234" t="s">
         <v>48</v>
       </c>
-      <c r="D50" s="210"/>
-      <c r="E50" s="210"/>
-      <c r="F50" s="210"/>
-      <c r="G50" s="210"/>
-      <c r="H50" s="210"/>
-      <c r="I50" s="210"/>
-      <c r="J50" s="210"/>
-      <c r="K50" s="210"/>
-      <c r="L50" s="210"/>
+      <c r="D50" s="235"/>
+      <c r="E50" s="235"/>
+      <c r="F50" s="235"/>
+      <c r="G50" s="235"/>
+      <c r="H50" s="235"/>
+      <c r="I50" s="235"/>
+      <c r="J50" s="235"/>
+      <c r="K50" s="235"/>
+      <c r="L50" s="235"/>
       <c r="M50" s="98"/>
       <c r="N50" s="21"/>
       <c r="O50" s="3"/>
@@ -7622,7 +7621,7 @@
       <c r="BF57" s="5"/>
       <c r="BG57" s="6"/>
     </row>
-    <row r="58" spans="1:59" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:59" ht="19" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="2"/>
       <c r="B58" s="121" t="s">
         <v>19</v>
@@ -7703,7 +7702,7 @@
       <c r="BF58" s="5"/>
       <c r="BG58" s="6"/>
     </row>
-    <row r="59" spans="1:59" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:59" ht="19" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="2"/>
       <c r="B59" s="121" t="s">
         <v>20</v>
@@ -7784,7 +7783,7 @@
       <c r="BF59" s="5"/>
       <c r="BG59" s="6"/>
     </row>
-    <row r="60" spans="1:59" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:59" ht="19" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="2"/>
       <c r="B60" s="121" t="s">
         <v>21</v>
@@ -7864,7 +7863,7 @@
       <c r="BF60" s="5"/>
       <c r="BG60" s="6"/>
     </row>
-    <row r="61" spans="1:59" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:59" ht="19" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="2"/>
       <c r="B61" s="121" t="s">
         <v>22</v>
@@ -8386,7 +8385,7 @@
       <c r="BF67" s="5"/>
       <c r="BG67" s="6"/>
     </row>
-    <row r="68" spans="1:59" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:59" ht="18.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="2"/>
       <c r="B68" s="121" t="s">
         <v>22</v>
@@ -8464,7 +8463,7 @@
       <c r="BF68" s="5"/>
       <c r="BG68" s="6"/>
     </row>
-    <row r="69" spans="1:59" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:59" ht="18.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="2"/>
       <c r="B69" s="121" t="s">
         <v>23</v>
@@ -8529,23 +8528,23 @@
       <c r="BF69" s="5"/>
       <c r="BG69" s="6"/>
     </row>
-    <row r="70" spans="1:59" ht="16" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:59" ht="16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" s="2"/>
       <c r="B70" s="127"/>
       <c r="C70" s="120" t="s">
         <v>66</v>
       </c>
-      <c r="D70" s="211" t="s">
+      <c r="D70" s="236" t="s">
         <v>88</v>
       </c>
-      <c r="E70" s="212"/>
-      <c r="F70" s="212"/>
-      <c r="G70" s="212"/>
-      <c r="H70" s="212"/>
-      <c r="I70" s="212"/>
-      <c r="J70" s="212"/>
-      <c r="K70" s="212"/>
-      <c r="L70" s="212"/>
+      <c r="E70" s="237"/>
+      <c r="F70" s="237"/>
+      <c r="G70" s="237"/>
+      <c r="H70" s="237"/>
+      <c r="I70" s="237"/>
+      <c r="J70" s="237"/>
+      <c r="K70" s="237"/>
+      <c r="L70" s="237"/>
       <c r="M70" s="17"/>
       <c r="N70" s="21"/>
       <c r="O70" s="95"/>
@@ -8607,23 +8606,23 @@
       <c r="BF70" s="5"/>
       <c r="BG70" s="6"/>
     </row>
-    <row r="71" spans="1:59" ht="16" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:59" ht="16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" s="2"/>
       <c r="B71" s="127"/>
       <c r="C71" s="120" t="s">
         <v>67</v>
       </c>
-      <c r="D71" s="211" t="s">
+      <c r="D71" s="236" t="s">
         <v>89</v>
       </c>
-      <c r="E71" s="212"/>
-      <c r="F71" s="212"/>
-      <c r="G71" s="212"/>
-      <c r="H71" s="212"/>
-      <c r="I71" s="212"/>
-      <c r="J71" s="212"/>
-      <c r="K71" s="212"/>
-      <c r="L71" s="212"/>
+      <c r="E71" s="237"/>
+      <c r="F71" s="237"/>
+      <c r="G71" s="237"/>
+      <c r="H71" s="237"/>
+      <c r="I71" s="237"/>
+      <c r="J71" s="237"/>
+      <c r="K71" s="237"/>
+      <c r="L71" s="237"/>
       <c r="M71" s="17"/>
       <c r="N71" s="21"/>
       <c r="O71" s="95"/>
@@ -8691,17 +8690,17 @@
       <c r="C72" s="120" t="s">
         <v>68</v>
       </c>
-      <c r="D72" s="211" t="s">
+      <c r="D72" s="236" t="s">
         <v>90</v>
       </c>
-      <c r="E72" s="211"/>
-      <c r="F72" s="211"/>
-      <c r="G72" s="211"/>
-      <c r="H72" s="211"/>
-      <c r="I72" s="211"/>
-      <c r="J72" s="211"/>
-      <c r="K72" s="211"/>
-      <c r="L72" s="211"/>
+      <c r="E72" s="236"/>
+      <c r="F72" s="236"/>
+      <c r="G72" s="236"/>
+      <c r="H72" s="236"/>
+      <c r="I72" s="236"/>
+      <c r="J72" s="236"/>
+      <c r="K72" s="236"/>
+      <c r="L72" s="236"/>
       <c r="M72" s="17"/>
       <c r="N72" s="21"/>
       <c r="O72" s="95"/>
@@ -8769,17 +8768,17 @@
       <c r="C73" s="120" t="s">
         <v>69</v>
       </c>
-      <c r="D73" s="211" t="s">
+      <c r="D73" s="236" t="s">
         <v>91</v>
       </c>
-      <c r="E73" s="211"/>
-      <c r="F73" s="211"/>
-      <c r="G73" s="211"/>
-      <c r="H73" s="211"/>
-      <c r="I73" s="211"/>
-      <c r="J73" s="211"/>
-      <c r="K73" s="211"/>
-      <c r="L73" s="211"/>
+      <c r="E73" s="236"/>
+      <c r="F73" s="236"/>
+      <c r="G73" s="236"/>
+      <c r="H73" s="236"/>
+      <c r="I73" s="236"/>
+      <c r="J73" s="236"/>
+      <c r="K73" s="236"/>
+      <c r="L73" s="236"/>
       <c r="M73" s="17"/>
       <c r="N73" s="21"/>
       <c r="O73" s="95"/>
@@ -8847,17 +8846,17 @@
       <c r="C74" s="120" t="s">
         <v>103</v>
       </c>
-      <c r="D74" s="211" t="s">
+      <c r="D74" s="236" t="s">
         <v>106</v>
       </c>
-      <c r="E74" s="211"/>
-      <c r="F74" s="211"/>
-      <c r="G74" s="211"/>
-      <c r="H74" s="211"/>
-      <c r="I74" s="211"/>
-      <c r="J74" s="211"/>
-      <c r="K74" s="211"/>
-      <c r="L74" s="211"/>
+      <c r="E74" s="236"/>
+      <c r="F74" s="236"/>
+      <c r="G74" s="236"/>
+      <c r="H74" s="236"/>
+      <c r="I74" s="236"/>
+      <c r="J74" s="236"/>
+      <c r="K74" s="236"/>
+      <c r="L74" s="236"/>
       <c r="M74" s="17"/>
       <c r="N74" s="21"/>
       <c r="O74" s="95"/>
@@ -8925,17 +8924,17 @@
       <c r="C75" s="120" t="s">
         <v>104</v>
       </c>
-      <c r="D75" s="211" t="s">
+      <c r="D75" s="236" t="s">
         <v>105</v>
       </c>
-      <c r="E75" s="211"/>
-      <c r="F75" s="211"/>
-      <c r="G75" s="211"/>
-      <c r="H75" s="211"/>
-      <c r="I75" s="211"/>
-      <c r="J75" s="211"/>
-      <c r="K75" s="211"/>
-      <c r="L75" s="211"/>
+      <c r="E75" s="236"/>
+      <c r="F75" s="236"/>
+      <c r="G75" s="236"/>
+      <c r="H75" s="236"/>
+      <c r="I75" s="236"/>
+      <c r="J75" s="236"/>
+      <c r="K75" s="236"/>
+      <c r="L75" s="236"/>
       <c r="M75" s="17"/>
       <c r="N75" s="21"/>
       <c r="O75" s="95"/>
@@ -8997,7 +8996,7 @@
       <c r="BF75" s="5"/>
       <c r="BG75" s="6"/>
     </row>
-    <row r="76" spans="1:59" ht="16" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:59" ht="16" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" s="2"/>
       <c r="B76" s="127"/>
       <c r="C76" s="128"/>
@@ -9214,7 +9213,7 @@
       <c r="BF78" s="5"/>
       <c r="BG78" s="6"/>
     </row>
-    <row r="79" spans="1:59" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:59" ht="18.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="2"/>
       <c r="B79" s="121" t="s">
         <v>93</v>
@@ -9222,15 +9221,15 @@
       <c r="C79" s="161" t="s">
         <v>71</v>
       </c>
-      <c r="D79" s="203"/>
-      <c r="E79" s="204"/>
-      <c r="F79" s="204"/>
-      <c r="G79" s="204"/>
-      <c r="H79" s="204"/>
-      <c r="I79" s="204"/>
-      <c r="J79" s="204"/>
-      <c r="K79" s="204"/>
-      <c r="L79" s="204"/>
+      <c r="D79" s="232"/>
+      <c r="E79" s="233"/>
+      <c r="F79" s="233"/>
+      <c r="G79" s="233"/>
+      <c r="H79" s="233"/>
+      <c r="I79" s="233"/>
+      <c r="J79" s="233"/>
+      <c r="K79" s="233"/>
+      <c r="L79" s="233"/>
       <c r="M79" s="17"/>
       <c r="N79" s="21"/>
       <c r="O79" s="95"/>
@@ -9292,7 +9291,7 @@
       <c r="BF79" s="3"/>
       <c r="BG79" s="16"/>
     </row>
-    <row r="80" spans="1:59" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:59" ht="18.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="2"/>
       <c r="B80" s="121" t="s">
         <v>94</v>
@@ -9300,15 +9299,15 @@
       <c r="C80" s="161" t="s">
         <v>71</v>
       </c>
-      <c r="D80" s="203"/>
-      <c r="E80" s="204"/>
-      <c r="F80" s="204"/>
-      <c r="G80" s="204"/>
-      <c r="H80" s="204"/>
-      <c r="I80" s="204"/>
-      <c r="J80" s="204"/>
-      <c r="K80" s="204"/>
-      <c r="L80" s="204"/>
+      <c r="D80" s="232"/>
+      <c r="E80" s="233"/>
+      <c r="F80" s="233"/>
+      <c r="G80" s="233"/>
+      <c r="H80" s="233"/>
+      <c r="I80" s="233"/>
+      <c r="J80" s="233"/>
+      <c r="K80" s="233"/>
+      <c r="L80" s="233"/>
       <c r="M80" s="17"/>
       <c r="N80" s="21"/>
       <c r="O80" s="95"/>
@@ -11100,31 +11099,6 @@
     </row>
   </sheetData>
   <mergeCells count="39">
-    <mergeCell ref="E4:K4"/>
-    <mergeCell ref="E2:K2"/>
-    <mergeCell ref="U2:AG2"/>
-    <mergeCell ref="V7:Z7"/>
-    <mergeCell ref="AC7:AG7"/>
-    <mergeCell ref="AM7:AO7"/>
-    <mergeCell ref="AU7:AW7"/>
-    <mergeCell ref="V4:X4"/>
-    <mergeCell ref="AU4:AW4"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="B19:D19"/>
-    <mergeCell ref="B30:F30"/>
-    <mergeCell ref="Q7:S7"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="C9:F9"/>
-    <mergeCell ref="O9:O10"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="AS9:AS10"/>
-    <mergeCell ref="AZ9:AZ10"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="AK9:AK10"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="AA4:AC4"/>
-    <mergeCell ref="AE4:AG4"/>
     <mergeCell ref="D79:L79"/>
     <mergeCell ref="D80:L80"/>
     <mergeCell ref="B47:F47"/>
@@ -11137,8 +11111,33 @@
     <mergeCell ref="C48:L48"/>
     <mergeCell ref="D74:L74"/>
     <mergeCell ref="D75:L75"/>
+    <mergeCell ref="AZ9:AZ10"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="AK9:AK10"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="AA4:AC4"/>
+    <mergeCell ref="AE4:AG4"/>
     <mergeCell ref="V9:V10"/>
     <mergeCell ref="AC9:AC10"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="B30:F30"/>
+    <mergeCell ref="Q7:S7"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="C9:F9"/>
+    <mergeCell ref="O9:O10"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="AM7:AO7"/>
+    <mergeCell ref="AU7:AW7"/>
+    <mergeCell ref="V4:X4"/>
+    <mergeCell ref="AU4:AW4"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="AS9:AS10"/>
+    <mergeCell ref="E4:K4"/>
+    <mergeCell ref="E2:K2"/>
+    <mergeCell ref="U2:AG2"/>
+    <mergeCell ref="V7:Z7"/>
+    <mergeCell ref="AC7:AG7"/>
   </mergeCells>
   <conditionalFormatting sqref="AM18:AQ18 AU18:AY18 S18:V19 Y18:AC19 AF18:AI19 AK19 AN19:AQ19 AS19 AV19:AY19 T20:U25 Y20:Y25 AA20:AB25 AF20:AF25 AH20:AI25 AN20:AN25 AP20:AQ25 AV20:AV25 AX20:AY25 S26:V29 Y26:AC29 AF26:AI29 AM26:AQ29 AU26:AY29 U52:V57 Y52:Y57 AB52:AC57 AF52:AF57 AI52:AI57 AM52:AN57 AQ52:AQ57 AU52:AV57 U83:V85 Y83:Y85 AI83:AI86 AM83:AN86 AQ83:AQ86 AU83:AV86 U90:V90 Y90 AB83:AC90 AF83:AF90 AI88:AI90 AM88:AN90 AQ88:AQ90 AU88:AV90 S91:V91 Y91:AC91 AF91:AI91 AM91:AQ91 AU91:AX91 AI92">
     <cfRule type="cellIs" dxfId="0" priority="1" stopIfTrue="1" operator="lessThan">

</xml_diff>